<commit_message>
P1(영역2): enterprise v19 전술 분리 — 은닉(ST)·방어 무력화(DM)(v3)
ATT&CK v19(2026-04) 방어 회피 분리를 반영(D15). 구 방어 회피(DE) 8행을
은닉(ST, TA0005 유지) 6행·방어 무력화(DM, 신설 TA0112) 2행으로 재코딩.

- ENT-DE-* → ENT-ST-*(지표 삭제·위장·난독화·인메모리·루트킷·펌웨어)
  / ENT-DM-*(EDR 무력화 BYOVD·취약 드라이버 로드)
- 전술 12→13: DOMAIN_ORDER·TACTICS·frameworks 어휘 갱신
- text DE.yaml → ST.yaml·DM.yaml 분리, 사고 매핑·시나리오 전술 라벨 갱신
- 저장소 v19.2 추출본 전술 배정과 대조(이벤트 로그 삭제 T1685.005만
  v19 DM이나 흔적 제거 목적이라 ST 행에 함께 매핑)
- 세부위협 51행 불변, 검증 오류·경고 0, v2·v5 빌드 정상

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RuSCf1v2AwGLbjYwwieALL
</commit_message>
<xml_diff>
--- a/enterprise/output/통합_고도화엔터프라이즈_보안위협_매트릭스_v2.xlsx
+++ b/enterprise/output/통합_고도화엔터프라이즈_보안위협_매트릭스_v2.xlsx
@@ -782,7 +782,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>ATT&amp;CK Enterprise 침투~영향 12개 — [IA]초기 침투 → [EX]실행 → [PE]지속 → [PV]권한 상승 → [DE]방어 회피 → [CA]자격증명 접근 → [DI]탐색 → [LM]측면 이동 → [CO]수집 → [C2]명령·제어 → [EF]반출 → [IM]영향</t>
+          <t>ATT&amp;CK Enterprise 침투~영향 13개(v19 방어 회피 분리) — [IA]초기 침투 → [EX]실행 → [PE]지속 → [PV]권한 상승 → [ST]은닉 → [DM]방어 무력화 → [CA]자격증명 접근 → [DI]탐색 → [LM]측면 이동 → [CO]수집 → [C2]명령·제어 → [EF]반출 → [IM]영향</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>51개 / 위협분류 46 / 전술 12</t>
+          <t>51개 / 위협분류 46 / 전술 13</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
 5. ENT-IM-02 복구 방해(섀도 카피·백업 삭제) — 매우 높음, 실제 사고 2건(EDR·XDR)
 6. ENT-LM-04 원격 서비스 취약점 악용(웜 확산) — 매우 높음, 실제 사고 2건(EDR·XDR)
 7. ENT-IA-01 인터넷 노출 경계·엣지 장비 취약점 악용(빠른 n-day·0-day) — 높음, 실제 사고 10건(행위·네트워크·아이덴티티)
-8. ENT-DE-01.1 보안 도구 무력화(EDR 변조·BYOVD EDR 킬러) — 높음, 실제 사고 7건(행위·네트워크·아이덴티티)
+8. ENT-DM-01.1 보안 도구 무력화(EDR 변조·BYOVD EDR 킬러) — 높음, 실제 사고 7건(행위·네트워크·아이덴티티)
 9. ENT-LM-01 원격 서비스 악용(RDP·SMB·WinRM) — 높음, 실제 사고 5건(행위·네트워크·아이덴티티)
 10. ENT-IA-02 외부 원격 서비스 악용(VPN·RDP·원격 관리) — 높음, 실제 사고 4건(행위·네트워크·아이덴티티)</t>
         </is>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-07</t>
+          <t>ENT-ST-05</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr"/>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-05</t>
+          <t>ENT-ST-03</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr"/>
@@ -1570,7 +1570,7 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-04</t>
+          <t>ENT-ST-02</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr"/>
@@ -1868,7 +1868,7 @@
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-03</t>
+          <t>ENT-ST-01</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr"/>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-03</t>
+          <t>ENT-ST-01</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr"/>
@@ -2696,7 +2696,7 @@
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-08</t>
+          <t>ENT-ST-06</t>
         </is>
       </c>
       <c r="G51" s="9" t="inlineStr"/>
@@ -2725,7 +2725,7 @@
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>ENT-PE-01, ENT-DE-01.2</t>
+          <t>ENT-PE-01, ENT-DM-01.2</t>
         </is>
       </c>
       <c r="G52" s="9" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-06</t>
+          <t>ENT-ST-04</t>
         </is>
       </c>
       <c r="G65" s="9" t="inlineStr"/>
@@ -3164,7 +3164,7 @@
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-01.1</t>
+          <t>ENT-DM-01.1</t>
         </is>
       </c>
       <c r="G67" s="9" t="inlineStr">
@@ -3197,7 +3197,7 @@
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-03</t>
+          <t>ENT-ST-01</t>
         </is>
       </c>
       <c r="G68" s="9" t="inlineStr"/>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-03, ENT-DI-02, ENT-C2-01.2, ENT-DI-01, ENT-EF-01, ENT-C2-01.1, ENT-EX-01.2, ENT-C2-06, ENT-PE-03, ENT-PE-01, ENT-PE-04</t>
+          <t>ENT-ST-01, ENT-DI-02, ENT-C2-01.2, ENT-DI-01, ENT-EF-01, ENT-C2-01.1, ENT-EX-01.2, ENT-C2-06, ENT-PE-03, ENT-PE-01, ENT-PE-04</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-03</t>
+          <t>ENT-ST-01</t>
         </is>
       </c>
     </row>
@@ -3430,7 +3430,7 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-01.1, ENT-DE-01.2, ENT-EX-01.1, ENT-EX-03, ENT-DE-08, ENT-EX-01.2, ENT-EX-04, ENT-PE-03, ENT-PE-01, ENT-PV-03, ENT-PE-02</t>
+          <t>ENT-DM-01.1, ENT-DM-01.2, ENT-EX-01.1, ENT-EX-03, ENT-ST-06, ENT-EX-01.2, ENT-EX-04, ENT-PE-03, ENT-PE-01, ENT-PV-03, ENT-PE-02</t>
         </is>
       </c>
     </row>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>ENT-EX-01.1, ENT-C2-05, ENT-PV-01.1, ENT-IA-04, ENT-DE-06, ENT-DE-05, ENT-IA-03</t>
+          <t>ENT-EX-01.1, ENT-C2-05, ENT-PV-01.1, ENT-IA-04, ENT-ST-04, ENT-ST-03, ENT-IA-03</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3706,7 @@
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>ENT-IM-01, ENT-IM-05, ENT-EF-02, ENT-IA-05, ENT-IM-02, ENT-IA-01, ENT-DE-01.1, ENT-LM-01, ENT-IA-02, ENT-CA-01.1, ENT-DE-01.2, ENT-DE-03, ENT-EX-01.1, ENT-DI-02, ENT-LM-02, ENT-C2-01.2, ENT-IM-03, ENT-DI-01, ENT-C2-05, ENT-EF-01, ENT-C2-04, ENT-C2-01.1, ENT-CA-03, ENT-EX-03, ENT-PV-01.1, ENT-IM-04, ENT-LM-03, ENT-PV-04, ENT-EX-01.2, ENT-C2-06, ENT-C2-03, ENT-DE-06, ENT-DE-07, ENT-EX-04, ENT-CO-01, ENT-PE-03, ENT-DE-05, ENT-CA-04, ENT-PE-01, ENT-CO-02, ENT-PV-03, ENT-DE-04, ENT-IA-03, ENT-DI-03, ENT-PV-01.2, ENT-PE-02, ENT-CA-01.2</t>
+          <t>ENT-IM-01, ENT-IM-05, ENT-EF-02, ENT-IA-05, ENT-IM-02, ENT-IA-01, ENT-DM-01.1, ENT-LM-01, ENT-IA-02, ENT-CA-01.1, ENT-DM-01.2, ENT-ST-01, ENT-EX-01.1, ENT-DI-02, ENT-LM-02, ENT-C2-01.2, ENT-IM-03, ENT-DI-01, ENT-C2-05, ENT-EF-01, ENT-C2-04, ENT-C2-01.1, ENT-CA-03, ENT-EX-03, ENT-PV-01.1, ENT-IM-04, ENT-LM-03, ENT-PV-04, ENT-EX-01.2, ENT-C2-06, ENT-C2-03, ENT-ST-04, ENT-ST-05, ENT-EX-04, ENT-CO-01, ENT-PE-03, ENT-ST-03, ENT-CA-04, ENT-PE-01, ENT-CO-02, ENT-PV-03, ENT-ST-02, ENT-IA-03, ENT-DI-03, ENT-PV-01.2, ENT-PE-02, ENT-CA-01.2</t>
         </is>
       </c>
     </row>
@@ -3729,7 +3729,7 @@
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-01.1, ENT-DE-01.2, ENT-IM-03, ENT-EX-03, ENT-DE-08, ENT-DE-07, ENT-DE-04, ENT-PE-02</t>
+          <t>ENT-DM-01.1, ENT-DM-01.2, ENT-IM-03, ENT-EX-03, ENT-ST-06, ENT-ST-05, ENT-ST-02, ENT-PE-02</t>
         </is>
       </c>
     </row>
@@ -3879,12 +3879,12 @@
       </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>IA · EX · PE · PV · DE · CA · DI · LM · CO · C2 · EF · IM</t>
+          <t>IA · EX · PE · PV · ST · DM · CA · DI · LM · CO · C2 · EF · IM</t>
         </is>
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>ENT-IA-02, ENT-IA-03, ENT-IA-04, ENT-IA-05, ENT-EX-01.1, ENT-EX-01.2, ENT-EX-03, ENT-EX-04, ENT-PE-01, ENT-PE-02, ENT-PE-03, ENT-PE-04, ENT-PV-01.1, ENT-PV-01.2, ENT-PV-03, ENT-DE-03, ENT-DE-04, ENT-DE-05, ENT-DE-06, ENT-DE-07, ENT-DE-08, ENT-CA-01.1, ENT-CA-01.2, ENT-CA-03, ENT-CA-04, ENT-DI-01, ENT-DI-02, ENT-DI-03, ENT-LM-01, ENT-LM-02, ENT-LM-03, ENT-LM-04, ENT-CO-01, ENT-CO-02, ENT-C2-01.1, ENT-C2-01.2, ENT-C2-03, ENT-C2-04, ENT-C2-05, ENT-C2-06, ENT-EF-01, ENT-EF-02, ENT-IM-01, ENT-IM-02, ENT-IM-03, ENT-IM-04, ENT-IM-05</t>
+          <t>ENT-IA-02, ENT-IA-03, ENT-IA-04, ENT-IA-05, ENT-EX-01.1, ENT-EX-01.2, ENT-EX-03, ENT-EX-04, ENT-PE-01, ENT-PE-02, ENT-PE-03, ENT-PE-04, ENT-PV-01.1, ENT-PV-01.2, ENT-PV-03, ENT-ST-01, ENT-ST-02, ENT-ST-03, ENT-ST-04, ENT-ST-05, ENT-ST-06, ENT-CA-01.1, ENT-CA-01.2, ENT-CA-03, ENT-CA-04, ENT-DI-01, ENT-DI-02, ENT-DI-03, ENT-LM-01, ENT-LM-02, ENT-LM-03, ENT-LM-04, ENT-CO-01, ENT-CO-02, ENT-C2-01.1, ENT-C2-01.2, ENT-C2-03, ENT-C2-04, ENT-C2-05, ENT-C2-06, ENT-EF-01, ENT-EF-02, ENT-IM-01, ENT-IM-02, ENT-IM-03, ENT-IM-04, ENT-IM-05</t>
         </is>
       </c>
       <c r="I2" s="9" t="inlineStr">
@@ -4003,12 +4003,12 @@
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>DM</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-01.1</t>
+          <t>ENT-DM-01.1</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
@@ -4189,12 +4189,12 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>PV · DE</t>
+          <t>PV · DM</t>
         </is>
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>ENT-PV-04, ENT-DE-01.1, ENT-DE-01.2</t>
+          <t>ENT-PV-04, ENT-DM-01.1, ENT-DM-01.2</t>
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>호스트·엔드포인트·네트워크·C2·방어 회피·온프레미스 AD 인접 기법만. 클라우드·신원·OT·AI·공급망 특화는 통합 v4.1 요약 ID로 연계만</t>
+          <t>호스트·엔드포인트·네트워크·C2·은닉·방어 무력화·온프레미스 AD 인접 기법만. 클라우드·신원·OT·AI·공급망 특화는 통합 v4.1 요약 ID로 연계만</t>
         </is>
       </c>
     </row>
@@ -5035,7 +5035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5091,61 +5091,61 @@
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>평가</t>
+          <t>구조</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>빈발 지수·심각도 영향만·사고 정리(P1b·P2·P3)</t>
+          <t>v19 전술 분리 — 은닉·방어 무력화(P1)</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>편재 기법(LOLBin·WMI·Kerberoasting·UAC·지표 삭제·DNS/웹 C2·스테이징 등) 기법 일반 서술 9건을 사고 DB에서 제거하고 ATT&amp;CK 절차 수 기반 '빈발 지수'(≥100 상·≥30 중)로 발생가능성에 반영. Cobalt Strike(Operation MORPHEUS)·UEFI 임플란트(LoJax·MoonBounce)·Gamaredon USB·CISA #StopRansomware 4건은 실제 사례로 재구성. ATT&amp;CK 주체 수 하위 기법 롤업 버그 수정, BYOVD 매핑 정정(T1547.006 Linux 전용 제거→T1685·T1543.003). 심각도는 영향만으로 재판정(엔에이블러 상 26→8). 발생가능성 상에 서로 다른 행위자·캠페인 2개 요건, 경계 플래그 신설. 사고 33→24, 위험도 매우 높음 6·높음 15·보통 25·낮음 5</t>
+          <t>ATT&amp;CK v19(2026-04)의 방어 회피 분리를 반영(D15) — 구 방어 회피(DE) 8행을 은닉(ST, TA0005 유지) 6행·방어 무력화(DM, 신설 TA0112) 2행으로 재코딩. ENT-DE-* → ENT-ST-*(지표 삭제·위장·난독화·인메모리·루트킷·펌웨어)·ENT-DM-*(EDR 무력화 BYOVD·취약 드라이버 로드). 전술 12→13, DOMAIN_ORDER·TACTICS·frameworks 어휘·text(ST.yaml·DM.yaml 신설, DE.yaml 제거)·사고 매핑·시나리오 전술 라벨 일괄 갱신. 저장소 ATT&amp;CK v19.2 추출본 전술 배정과 대조(이벤트 로그 삭제 T1685.005만 v19 DM이나 흔적 제거 목적이라 ST 행에 함께 매핑). 세부위협 51행·검증 오류·경고 0 유지</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>검토 5.1~5.4·6.1 — 근거 무결성·렌즈 변별력 교정</t>
+          <t>검토 D15 — ATT&amp;CK v19.2 전술 체계 반영</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>구조</t>
+          <t>평가</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>워크북·CSV(scripts/build_enterprise_threat_matrix.py)</t>
+          <t>빈발 지수·심각도 영향만·사고 정리(P1b·P2·P3)</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>15시트 워크북·CSV 생성(세부위협 51행). aiattack 빌드를 이식하되 레거시 공백·요구 방어 수준 고유 축 시트와 ATT&amp;CK·KEV 교차 시트를 둠. 위험도 매우 높음 17·높음 12·보통 21·낮음 1, 근거 수준 실제 사고 45·ATT&amp;CK/KEV 다수 3·일부 2·이론 1. 우선순위에 요구 방어 수준(방어 난이도)·ATT&amp;CK 주체 수 보조(D5). 빌드 전 검증기 자동 실행</t>
+          <t>편재 기법(LOLBin·WMI·Kerberoasting·UAC·지표 삭제·DNS/웹 C2·스테이징 등) 기법 일반 서술 9건을 사고 DB에서 제거하고 ATT&amp;CK 절차 수 기반 '빈발 지수'(≥100 상·≥30 중)로 발생가능성에 반영. Cobalt Strike(Operation MORPHEUS)·UEFI 임플란트(LoJax·MoonBounce)·Gamaredon USB·CISA #StopRansomware 4건은 실제 사례로 재구성. ATT&amp;CK 주체 수 하위 기법 롤업 버그 수정, BYOVD 매핑 정정(T1547.006 Linux 전용 제거→T1685·T1543.003). 심각도는 영향만으로 재판정(엔에이블러 상 26→8). 발생가능성 상에 서로 다른 행위자·캠페인 2개 요건, 경계 플래그 신설. 사고 33→24, 위험도 매우 높음 6·높음 15·보통 25·낮음 5</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>②단계(v1) — 분류·근거·평가를 한 워크북에서 검토</t>
+          <t>검토 5.1~5.4·6.1 — 근거 무결성·렌즈 변별력 교정</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
@@ -5155,22 +5155,22 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>문구</t>
+          <t>구조</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>관점 문구(data/text/*.yaml)</t>
+          <t>워크북·CSV(scripts/build_enterprise_threat_matrix.py)</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>51개 행 전부에 핵심 요약·요약설명·참조(■ 관점·■ 실제 사례)·탐지·대응 작성. 인용 사례 83건([실제 사고]·[정부 경보]·[실증]), 실제 사고가 없는 5개 행(드라이브바이·네이티브 API·계정 조작·캐시 자격증명·보안 SW 탐색)은 '공개 사고 미확인 — 사유'로 표기. 가드레일 D11(공세 제작법 미기재, 탐지·대응 중심) 적용</t>
+          <t>15시트 워크북·CSV 생성(세부위협 51행). aiattack 빌드를 이식하되 레거시 공백·요구 방어 수준 고유 축 시트와 ATT&amp;CK·KEV 교차 시트를 둠. 위험도 매우 높음 17·높음 12·보통 21·낮음 1, 근거 수준 실제 사고 45·ATT&amp;CK/KEV 다수 3·일부 2·이론 1. 우선순위에 요구 방어 수준(방어 난이도)·ATT&amp;CK 주체 수 보조(D5). 빌드 전 검증기 자동 실행</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>③단계(v2) — 방어 관점으로 행마다 근거·통제를 연결</t>
+          <t>②단계(v1) — 분류·근거·평가를 한 워크북에서 검토</t>
         </is>
       </c>
     </row>
@@ -5187,22 +5187,22 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>시나리오</t>
+          <t>문구</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>공격 체인 시나리오(data/scenarios.yaml)</t>
+          <t>관점 문구(data/text/*.yaml)</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>실제 사고를 침해 흐름 8개로 재구성(ESN-01~08) — 엣지 0-day→LotL→확산, 사람 운영 랜섬웨어(BYOVD·복구 방해), 파일전송 0-day 갈취(Cl0p), 웜 확산→파괴, 비콘 C2, MSP 신뢰 관계, 지표 삭제 은닉, 커널·펌웨어 하위 계층. 21개 단계·초크 포인트 16개</t>
+          <t>51개 행 전부에 핵심 요약·요약설명·참조(■ 관점·■ 실제 사례)·탐지·대응 작성. 인용 사례 83건([실제 사고]·[정부 경보]·[실증]), 실제 사고가 없는 5개 행(드라이브바이·네이티브 API·계정 조작·캐시 자격증명·보안 SW 탐색)은 '공개 사고 미확인 — 사유'로 표기. 가드레일 D11(공세 제작법 미기재, 탐지·대응 중심) 적용</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>한 행=한 행위로 나눈 세부위협을 흐름 안에서 보고 차단 지점을 드러냄</t>
+          <t>③단계(v2) — 방어 관점으로 행마다 근거·통제를 연결</t>
         </is>
       </c>
     </row>
@@ -5219,29 +5219,29 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>검증</t>
+          <t>시나리오</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>scripts/validate.py</t>
+          <t>공격 체인 시나리오(data/scenarios.yaml)</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>문구·시나리오 검사 이식 — 형식, 사례 라벨↔집계 상태·시점·수치 대조, 참조 ID(ATT&amp;CK·CVE↔KEV·NIST·연계) 존재·행 매핑, 가드레일. 문구 51·시나리오 8을 --strict로 검증해 오류·경고 0</t>
+          <t>실제 사고를 침해 흐름 8개로 재구성(ESN-01~08) — 엣지 0-day→LotL→확산, 사람 운영 랜섬웨어(BYOVD·복구 방해), 파일전송 0-day 갈취(Cl0p), 웜 확산→파괴, 비콘 C2, MSP 신뢰 관계, 지표 삭제 은닉, 커널·펌웨어 하위 계층. 21개 단계·초크 포인트 16개</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>문구·시나리오를 사고 DB·카탈로그와 기계적으로 대조</t>
+          <t>한 행=한 행위로 나눈 세부위협을 흐름 안에서 보고 차단 지점을 드러냄</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>v0</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
@@ -5251,22 +5251,22 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>결정</t>
+          <t>검증</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>작업방향 D5~D7·D9·D11·D12</t>
+          <t>scripts/validate.py</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>영역 2(고도화 엔터프라이즈 침해) 착수 결정 확정 — D5(ATT&amp;CK Enterprise에서 고도화·최근빈발·레거시난제 점수로 ~50행 선별, 자산 특화는 연계)·D6(Lv1 ATT&amp;CK 전술 + 레거시 공백 유형·요구 방어 수준 축)·D7(호스트·엔드포인트·네트워크·C2·회피·온프레미스 AD 인접, 클라우드·신원·OT·AI·공급망은 연계)·D9(통합본 뷰 Lv0)·D11(방어 자료 가드레일)·D12(v4.1 베이스라인)</t>
+          <t>문구·시나리오 검사 이식 — 형식, 사례 라벨↔집계 상태·시점·수치 대조, 참조 ID(ATT&amp;CK·CVE↔KEV·NIST·연계) 존재·행 매핑, 가드레일. 문구 51·시나리오 8을 --strict로 검증해 오류·경고 0</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>emerging/작업방향 10장 권장안을 영역 2 착수 결정으로 확정</t>
+          <t>문구·시나리오를 사고 DB·카탈로그와 기계적으로 대조</t>
         </is>
       </c>
     </row>
@@ -5283,22 +5283,22 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>구조</t>
+          <t>결정</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>분류 체계(data/taxonomy.yaml)</t>
+          <t>작업방향 D5~D7·D9·D11·D12</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>ATT&amp;CK Enterprise 침투~영향 12개 전술 도메인(IA·EX·PE·PV·DE·CA·DI·LM·CO·C2·EF·IM) → 위협분류 → 세부위협 51개 ID 대장(ENT-&lt;전술&gt;-NN). 전술 14개 중 정찰·자원 개발은 영역 1·정찰이 다뤄 제외·연계(D7). 행마다 레거시 방어 공백 유형·요구 방어 수준·주체·플랫폼·ATT&amp;CK·KEV·LOLBin·BYOVD 드라이버·대응 기준·연계·심각도. 심각도 상 26·중 24·하 1, 요구 방어 수준 '행위·네트워크·아이덴티티' 27·'EDR·XDR' 24</t>
+          <t>영역 2(고도화 엔터프라이즈 침해) 착수 결정 확정 — D5(ATT&amp;CK Enterprise에서 고도화·최근빈발·레거시난제 점수로 ~50행 선별, 자산 특화는 연계)·D6(Lv1 ATT&amp;CK 전술 + 레거시 공백 유형·요구 방어 수준 축)·D7(호스트·엔드포인트·네트워크·C2·회피·온프레미스 AD 인접, 클라우드·신원·OT·AI·공급망은 연계)·D9(통합본 뷰 Lv0)·D11(방어 자료 가드레일)·D12(v4.1 베이스라인)</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>D5·D6 확정안을 행 단위로 구현 — ①단계</t>
+          <t>emerging/작업방향 10장 권장안을 영역 2 착수 결정으로 확정</t>
         </is>
       </c>
     </row>
@@ -5315,22 +5315,22 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>근거</t>
+          <t>구조</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>사고 DB(data/incidents.yaml)</t>
+          <t>분류 체계(data/taxonomy.yaml)</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>고도화·레거시 우회 침해 사고 33건 구축 — 경계·엣지 0-day(Citrix Bleed·MOVEit·Fortinet·Ivanti·Cisco IOS XE·PAN-OS·ScreenConnect·Cleo), 국가배후 LotL(Volt Typhoon·APT28 Nearest Neighbor), 사람 운영 랜섬웨어(Black Basta·Scattered Spider·Akira·LockBit·RansomHub), BYOVD EDR 킬러, 웜 확산(NotPetya·WannaCry), 커널·펌웨어(BlackLotus·루트킷·펌웨어 임플란트), C2·DNS·이동식 매체. 실제 사고가 매핑된 세부위협 45/51. CVE는 KEV 목록과 대조</t>
+          <t>ATT&amp;CK Enterprise 침투~영향 12개 전술 도메인(IA·EX·PE·PV·DE·CA·DI·LM·CO·C2·EF·IM) → 위협분류 → 세부위협 51개 ID 대장(ENT-&lt;전술&gt;-NN). 전술 14개 중 정찰·자원 개발은 영역 1·정찰이 다뤄 제외·연계(D7). 행마다 레거시 방어 공백 유형·요구 방어 수준·주체·플랫폼·ATT&amp;CK·KEV·LOLBin·BYOVD 드라이버·대응 기준·연계·심각도. 심각도 상 26·중 24·하 1, 요구 방어 수준 '행위·네트워크·아이덴티티' 27·'EDR·XDR' 24</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>D8 — 호스트·엔드포인트·네트워크·랜섬웨어·엣지 0-day 사례로 근거 구축</t>
+          <t>D5·D6 확정안을 행 단위로 구현 — ①단계</t>
         </is>
       </c>
     </row>
@@ -5347,22 +5347,22 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>교차 매핑</t>
+          <t>근거</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>프레임워크·참고 문헌(data/frameworks.yaml)</t>
+          <t>사고 DB(data/incidents.yaml)</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>ATT&amp;CK Enterprise v19.2(1차 분류·근거), CISA KEV 2026.10.02(1,733건), LOLBAS 245·LOLDrivers 706, NIST SP 800-53 Rev.5, 참고 문헌 카탈로그 8종(ATT&amp;CK·KEV·CISA·Mandiant·LOLBAS·LOLDrivers·Hive·Securelist)</t>
+          <t>고도화·레거시 우회 침해 사고 33건 구축 — 경계·엣지 0-day(Citrix Bleed·MOVEit·Fortinet·Ivanti·Cisco IOS XE·PAN-OS·ScreenConnect·Cleo), 국가배후 LotL(Volt Typhoon·APT28 Nearest Neighbor), 사람 운영 랜섬웨어(Black Basta·Scattered Spider·Akira·LockBit·RansomHub), BYOVD EDR 킬러, 웜 확산(NotPetya·WannaCry), 커널·펌웨어(BlackLotus·루트킷·펌웨어 임플란트), C2·DNS·이동식 매체. 실제 사고가 매핑된 세부위협 45/51. CVE는 KEV 목록과 대조</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>역할별 교차 매핑·근거 출처와 이용 조건을 행 매핑 전에 고정</t>
+          <t>D8 — 호스트·엔드포인트·네트워크·랜섬웨어·엣지 0-day 사례로 근거 구축</t>
         </is>
       </c>
     </row>
@@ -5379,22 +5379,22 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>근거</t>
+          <t>교차 매핑</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>참조 추출본(reference/)</t>
+          <t>프레임워크·참고 문헌(data/frameworks.yaml)</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>ATT&amp;CK 추출본(prepare_attack.py — 기법 68·주체 977·절차 6,087, 절차 수는 최근빈발 신호), KEV 추출본(prepare_kev.py — 연도별 등재·경계/엣지 장비 비중 14~21%·같은 해 악용 비중), LOLBAS·LOLDrivers 추출본(prepare_lolbas.py), NIST·통합 v4.1 연계 ID 237개(prepare_refs.py)</t>
+          <t>ATT&amp;CK Enterprise v19.2(1차 분류·근거), CISA KEV 2026.10.02(1,733건), LOLBAS 245·LOLDrivers 706, NIST SP 800-53 Rev.5, 참고 문헌 카탈로그 8종(ATT&amp;CK·KEV·CISA·Mandiant·LOLBAS·LOLDrivers·Hive·Securelist)</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>빌드·검증을 저장소 안에서 재현. 겹치는 위협은 통합 v4.1 요약 ID로 연계만(D9)</t>
+          <t>역할별 교차 매핑·근거 출처와 이용 조건을 행 매핑 전에 고정</t>
         </is>
       </c>
     </row>
@@ -5411,20 +5411,52 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
+          <t>근거</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>참조 추출본(reference/)</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>ATT&amp;CK 추출본(prepare_attack.py — 기법 68·주체 977·절차 6,087, 절차 수는 최근빈발 신호), KEV 추출본(prepare_kev.py — 연도별 등재·경계/엣지 장비 비중 14~21%·같은 해 악용 비중), LOLBAS·LOLDrivers 추출본(prepare_lolbas.py), NIST·통합 v4.1 연계 ID 237개(prepare_refs.py)</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>빌드·검증을 저장소 안에서 재현. 겹치는 위협은 통합 v4.1 요약 ID로 연계만(D9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>v0</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
           <t>검증</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>scripts/validate.py · taxonomy_rules.py</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>검증기를 aiattack·물리 매트릭스 기준으로 이식 — 분류 체계 필드·어휘·ID 체계, ATT&amp;CK·KEV·NIST·연계·참고 문헌 키 존재, CVE↔KEV 대조, 레거시 공백·요구 방어 수준·주체·플랫폼 어휘, 사고 DB 필드·매핑·출처. 데이터 검증 오류·경고 0</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>①단계 완료 기준(매핑·참조 ID 전부 카탈로그에 존재, 검증 데이터 통과) 자동 확인</t>
         </is>
@@ -6019,12 +6051,12 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[DM] 방어 무력화</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>ENT-DE-01.1</t>
+          <t>ENT-DM-01.1</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -6275,12 +6307,12 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[DM] 방어 무력화</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>ENT-DE-01.2</t>
+          <t>ENT-DM-01.2</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
@@ -6339,12 +6371,12 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[ST] 은닉</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>ENT-DE-03</t>
+          <t>ENT-ST-01</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
@@ -7191,12 +7223,12 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[ST] 은닉</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>ENT-DE-08</t>
+          <t>ENT-ST-06</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
@@ -7771,12 +7803,12 @@
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[ST] 은닉</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>ENT-DE-06</t>
+          <t>ENT-ST-04</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
@@ -7835,12 +7867,12 @@
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[ST] 은닉</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>ENT-DE-07</t>
+          <t>ENT-ST-05</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
@@ -8091,12 +8123,12 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[ST] 은닉</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>ENT-DE-05</t>
+          <t>ENT-ST-03</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
@@ -8411,12 +8443,12 @@
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[ST] 은닉</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>ENT-DE-04</t>
+          <t>ENT-ST-02</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
@@ -8865,7 +8897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8880,6 +8912,7 @@
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8920,54 +8953,61 @@
       </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피
-Defense Evasion
-(8)</t>
+          <t>[ST] 은닉
+Stealth
+(6)</t>
         </is>
       </c>
       <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>[DM] 방어 무력화
+Defense Impairment
+(2)</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="inlineStr">
         <is>
           <t>[CA] 자격증명 접근
 Credential Access
 (4)</t>
         </is>
       </c>
-      <c r="G2" s="15" t="inlineStr">
+      <c r="H2" s="15" t="inlineStr">
         <is>
           <t>[DI] 탐색
 Discovery
 (3)</t>
         </is>
       </c>
-      <c r="H2" s="15" t="inlineStr">
+      <c r="I2" s="15" t="inlineStr">
         <is>
           <t>[LM] 측면 이동
 Lateral Movement
 (4)</t>
         </is>
       </c>
-      <c r="I2" s="15" t="inlineStr">
+      <c r="J2" s="15" t="inlineStr">
         <is>
           <t>[CO] 수집
 Collection
 (2)</t>
         </is>
       </c>
-      <c r="J2" s="15" t="inlineStr">
+      <c r="K2" s="15" t="inlineStr">
         <is>
           <t>[C2] 명령·제어
 Command and Control
 (6)</t>
         </is>
       </c>
-      <c r="K2" s="15" t="inlineStr">
+      <c r="L2" s="15" t="inlineStr">
         <is>
           <t>[EF] 반출
 Exfiltration
 (2)</t>
         </is>
       </c>
-      <c r="L2" s="15" t="inlineStr">
+      <c r="M2" s="15" t="inlineStr">
         <is>
           <t>[IM] 영향
 Impact
@@ -8998,40 +9038,45 @@
       </c>
       <c r="E3" s="17" t="inlineStr">
         <is>
-          <t>ENT-DE-01.1 보안 도구 무력화(EDR 변조·BYOVD EDR 킬러) [7]</t>
+          <t>ENT-ST-01 지표 삭제(이벤트 로그·파일 삭제) [2]</t>
         </is>
       </c>
       <c r="F3" s="17" t="inlineStr">
         <is>
+          <t>ENT-DM-01.1 보안 도구 무력화(EDR 변조·BYOVD EDR 킬러) [7]</t>
+        </is>
+      </c>
+      <c r="G3" s="17" t="inlineStr">
+        <is>
           <t>ENT-CA-01.1 OS 자격증명 덤프(LSASS 메모리) [4]</t>
         </is>
       </c>
-      <c r="G3" s="17" t="inlineStr">
+      <c r="H3" s="17" t="inlineStr">
         <is>
           <t>ENT-DI-02 도메인·AD 열거(계정·신뢰·공유) [2]</t>
         </is>
       </c>
-      <c r="H3" s="16" t="inlineStr">
+      <c r="I3" s="16" t="inlineStr">
         <is>
           <t>ENT-LM-04 원격 서비스 취약점 악용(웜 확산) [2]</t>
         </is>
       </c>
-      <c r="I3" s="18" t="inlineStr">
+      <c r="J3" s="18" t="inlineStr">
         <is>
           <t>ENT-CO-01 로컬·네트워크 공유 데이터 수집</t>
         </is>
       </c>
-      <c r="J3" s="17" t="inlineStr">
+      <c r="K3" s="17" t="inlineStr">
         <is>
           <t>ENT-C2-01.2 응용 계층 프로토콜(HTTPS) C2 [1]</t>
         </is>
       </c>
-      <c r="K3" s="16" t="inlineStr">
+      <c r="L3" s="16" t="inlineStr">
         <is>
           <t>ENT-EF-02 정상 웹 서비스·대체 프로토콜 경유 반출 [2]</t>
         </is>
       </c>
-      <c r="L3" s="16" t="inlineStr">
+      <c r="M3" s="16" t="inlineStr">
         <is>
           <t>ENT-IM-01 데이터 암호화(사람 운영 랜섬웨어) [8]</t>
         </is>
@@ -9058,42 +9103,47 @@
           <t>ENT-PV-04 권한 상승 취약점 악용(로컬·커널) [1]</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
-        <is>
-          <t>ENT-DE-01.2 취약·악성 드라이버 로드(커널) [3]</t>
-        </is>
-      </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>ENT-ST-06 펌웨어·부트킷(UEFI) 지속·은닉 [1]</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
+        <is>
+          <t>ENT-DM-01.2 취약·악성 드라이버 로드(커널) [3]</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>ENT-CA-03 Kerberoasting·AS-REP 로스팅 [1]</t>
         </is>
       </c>
-      <c r="G4" s="17" t="inlineStr">
+      <c r="H4" s="17" t="inlineStr">
         <is>
           <t>ENT-DI-01 호스트·시스템·네트워크 구성 탐색 [1]</t>
         </is>
       </c>
-      <c r="H4" s="17" t="inlineStr">
+      <c r="I4" s="17" t="inlineStr">
         <is>
           <t>ENT-LM-01 원격 서비스 악용(RDP·SMB·WinRM) [5]</t>
         </is>
       </c>
-      <c r="I4" s="18" t="inlineStr">
+      <c r="J4" s="18" t="inlineStr">
         <is>
           <t>ENT-CO-02 수집 데이터 압축·암호화 스테이징</t>
         </is>
       </c>
-      <c r="J4" s="17" t="inlineStr">
+      <c r="K4" s="17" t="inlineStr">
         <is>
           <t>ENT-C2-05 인그레스 도구 전송(페이로드 반입) [1]</t>
         </is>
       </c>
-      <c r="K4" s="17" t="inlineStr">
+      <c r="L4" s="17" t="inlineStr">
         <is>
           <t>ENT-EF-01 C2 채널 경유 반출</t>
         </is>
       </c>
-      <c r="L4" s="16" t="inlineStr">
+      <c r="M4" s="16" t="inlineStr">
         <is>
           <t>ENT-IM-02 복구 방해(섀도 카피·백업 삭제) [2]</t>
         </is>
@@ -9120,32 +9170,32 @@
           <t>ENT-PV-03 사용자 계정 컨트롤(UAC) 우회</t>
         </is>
       </c>
-      <c r="E5" s="17" t="inlineStr">
-        <is>
-          <t>ENT-DE-03 지표 삭제(이벤트 로그·파일 삭제) [2]</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>ENT-ST-02 위장(정상 이름·경로·서명 가장)</t>
+        </is>
+      </c>
+      <c r="G5" s="18" t="inlineStr">
         <is>
           <t>ENT-CA-04 입력 캡처·키로깅</t>
         </is>
       </c>
-      <c r="G5" s="19" t="inlineStr">
+      <c r="H5" s="19" t="inlineStr">
         <is>
           <t>ENT-DI-03 보안 소프트웨어·방어 환경 탐색</t>
         </is>
       </c>
-      <c r="H5" s="17" t="inlineStr">
+      <c r="I5" s="17" t="inlineStr">
         <is>
           <t>ENT-LM-02 대체 인증 자료 사용(Pass-the-Hash·Pass-the-Ticket) [2]</t>
         </is>
       </c>
-      <c r="J5" s="18" t="inlineStr">
+      <c r="K5" s="18" t="inlineStr">
         <is>
           <t>ENT-C2-01.1 암호화 채널·비표준/정상 포트 위장 C2 [1]</t>
         </is>
       </c>
-      <c r="L5" s="16" t="inlineStr">
+      <c r="M5" s="16" t="inlineStr">
         <is>
           <t>ENT-IM-05 금전 탈취·이중 협박 갈취 [2]</t>
         </is>
@@ -9174,25 +9224,25 @@
       </c>
       <c r="E6" s="18" t="inlineStr">
         <is>
-          <t>ENT-DE-08 펌웨어·부트킷(UEFI) 지속·은닉 [1]</t>
-        </is>
-      </c>
-      <c r="F6" s="19" t="inlineStr">
+          <t>ENT-ST-03 파일·정보 난독화·암호화</t>
+        </is>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
         <is>
           <t>ENT-CA-01.2 캐시된 도메인 자격증명 추출</t>
         </is>
       </c>
-      <c r="H6" s="18" t="inlineStr">
+      <c r="I6" s="18" t="inlineStr">
         <is>
           <t>ENT-LM-03 측면 도구 전송 [1]</t>
         </is>
       </c>
-      <c r="J6" s="18" t="inlineStr">
+      <c r="K6" s="18" t="inlineStr">
         <is>
           <t>ENT-C2-04 도메인 프런팅·다단계 프록시 [1]</t>
         </is>
       </c>
-      <c r="L6" s="17" t="inlineStr">
+      <c r="M6" s="17" t="inlineStr">
         <is>
           <t>ENT-IM-03 데이터 파괴·와이퍼 [1]</t>
         </is>
@@ -9206,15 +9256,15 @@
       </c>
       <c r="E7" s="18" t="inlineStr">
         <is>
-          <t>ENT-DE-04 위장(정상 이름·경로·서명 가장)</t>
-        </is>
-      </c>
-      <c r="J7" s="18" t="inlineStr">
+          <t>ENT-ST-04 인메모리·반사 코드 로딩</t>
+        </is>
+      </c>
+      <c r="K7" s="18" t="inlineStr">
         <is>
           <t>ENT-C2-03 정상 웹 서비스·클라우드 플랫폼 경유 C2</t>
         </is>
       </c>
-      <c r="L7" s="18" t="inlineStr">
+      <c r="M7" s="18" t="inlineStr">
         <is>
           <t>ENT-IM-04 서비스 중지·시스템 종료/재시작 [1]</t>
         </is>
@@ -9223,26 +9273,12 @@
     <row r="8">
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>ENT-DE-05 파일·정보 난독화·암호화</t>
-        </is>
-      </c>
-      <c r="J8" s="18" t="inlineStr">
+          <t>ENT-ST-05 루트킷(사용자·커널 은폐)</t>
+        </is>
+      </c>
+      <c r="K8" s="18" t="inlineStr">
         <is>
           <t>ENT-C2-06 DNS 경유 C2·터널링</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>ENT-DE-06 인메모리·반사 코드 로딩</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="E10" s="18" t="inlineStr">
-        <is>
-          <t>ENT-DE-07 루트킷(사용자·커널 은폐)</t>
         </is>
       </c>
     </row>
@@ -12295,38 +12331,38 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[ST] 은닉</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-01.1</t>
+          <t>ENT-ST-01</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>보안 도구 무력화·드라이버 로드</t>
+          <t>지표 삭제</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>보안 도구 무력화(EDR 변조·BYOVD EDR 킬러)</t>
+          <t>지표 삭제(이벤트 로그·파일 삭제)</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>서명된 취약 드라이버로 EDR·백신을 커널에서 무력화(BYOVD)</t>
+          <t>이벤트 로그·파일 삭제로 레거시 SIEM 탐지·분석 무력화</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>- 공격자는 서명된 취약 드라이버를 올려 EDR·백신을 커널에서 무력화할 수 있음
-- 보안 도구 자체가 꺼지므로 이후 단계가 전부 가려지고, 여러 랜섬웨어·국가배후가 EDR 킬러를 공유함</t>
+          <t>- 공격자는 이벤트 로그·파일을 지워 레거시 SIEM 탐지와 사후 분석을 무력화할 수 있음
+- 원격·불변 로그가 없으면 흔적이 사라져 추적이 어려워짐</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>Impair/disable security tools (EDR tampering, BYOVD killers)</t>
+          <t>Indicator removal (clear event logs, file deletion)</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr">
@@ -12336,7 +12372,7 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>커널·펌웨어 하위 계층 · 서명된 정상 도구 악용</t>
+          <t>시그니처 회피</t>
         </is>
       </c>
       <c r="J22" s="8" t="inlineStr">
@@ -12346,34 +12382,32 @@
       </c>
       <c r="K22" s="9" t="inlineStr">
         <is>
-          <t>랜섬웨어 · 국가배후</t>
+          <t>국가배후 · 랜섬웨어</t>
         </is>
       </c>
       <c r="L22" s="9" t="inlineStr">
         <is>
-          <t>Windows</t>
+          <t>Windows · Linux</t>
         </is>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>T1685</t>
+          <t>T1070, T1070.004, T1685.005</t>
         </is>
       </c>
       <c r="N22" s="9" t="inlineStr">
         <is>
-          <t>T1685 Disable or Modify Tools</t>
+          <t>T1070 Indicator Removal
+T1070.004 Indicator Removal: File Deletion
+T1685.005 Disable or Modify Tools: Clear Windows Event Logs</t>
         </is>
       </c>
       <c r="O22" s="8" t="n">
-        <v>155</v>
+        <v>335</v>
       </c>
       <c r="P22" s="8" t="inlineStr"/>
       <c r="Q22" s="8" t="inlineStr"/>
-      <c r="R22" s="8" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="R22" s="8" t="inlineStr"/>
       <c r="S22" s="9" t="inlineStr"/>
       <c r="T22" s="9" t="inlineStr"/>
       <c r="U22" s="9" t="inlineStr"/>
@@ -12397,26 +12431,26 @@
       </c>
       <c r="AB22" s="9" t="inlineStr"/>
       <c r="AC22" s="8" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="AD22" s="9" t="inlineStr">
         <is>
-          <t>실제 사고 7건(최근 3, 서로 다른 행위자·캠페인 7) · 빈발 지수 상(ATT&amp;CK 주체 155) · KEV - · 정부 경보 1 · 위협인텔 0 · 실증 0</t>
+          <t>실제 사고 2건(최근 1, 서로 다른 행위자·캠페인 2) · 빈발 지수 상(ATT&amp;CK 주체 335) · KEV - · 정부 경보 0 · 위협인텔 0 · 실증 0</t>
         </is>
       </c>
       <c r="AE22" s="9" t="inlineStr">
         <is>
-          <t>EDR·백신을 무력화해 이후 단계를 가리는 방어 무력화 수단 — 단독 피해보다 공격 성공률을 높이는 조건</t>
+          <t>이벤트 로그·파일을 지워 레거시 SIEM 탐지·사후 분석을 무력화 — 원격·불변 로그가 없으면 흔적이 사라짐(로그 삭제 T1685.005는 v19 방어 무력화로 재배치됐으나 공격 목적이 흔적 제거라 은닉 행으로 둠)</t>
         </is>
       </c>
       <c r="AF22" s="9" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AG22" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AH22" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI22" s="9" t="n">
         <v>0</v>
@@ -12428,73 +12462,70 @@
       </c>
       <c r="AK22" s="9" t="inlineStr">
         <is>
-          <t>ENI-012, ENI-013, ENI-015, ENI-016, ENI-017, ENI-036, ENI-037
-정부 경보: ENI-030</t>
+          <t>ENI-001, ENI-034</t>
         </is>
       </c>
       <c r="AL22" s="9" t="inlineStr">
         <is>
-          <t>랜섬·암호화 6 · 데이터 유출 2 · 자격증명·비밀 탈취 2 · 내부 접근 확보 2</t>
+          <t>내부 접근 확보 2 · 첩보·감시 1 · 측면 이동·확산 1 · 데이터 유출 1</t>
         </is>
       </c>
       <c r="AM22" s="9" t="inlineStr">
         <is>
-          <t>SI-4 System Monitoring
-SI-7 Software, Firmware, and Information Integrity
-CM-7 Least Functionality</t>
+          <t>AU-9 Protection of Audit Information
+SI-4 System Monitoring
+AU-6 Audit Record Review, Analysis, and Reporting</t>
         </is>
       </c>
       <c r="AN22" s="9" t="inlineStr">
         <is>
           <t>■ 탐지
-- 보안 서비스 중지·드라이버 로드와 EDR 텔레메트리 단절을 행위·네트워크 기반으로 탐지(NIST SI-4·SI-7)
+- 로그 삭제·감사 정책 변경 이벤트와 원격 수집 로그의 공백을 모니터링(NIST AU-6·SI-4)
 ■ 대응
-- 취약 드라이버 차단 목록(HVCI·블록리스트)·변조 방지와 보안 도구 상태를 중앙 감시(NIST SI-7·CM-7)
-- 참고: LOLDrivers 〈Project〉 · Hive Security 〈Modern Attack Techniques 2026〉</t>
+- 원격·불변 로그 전송과 로그 삭제 방지·보존 정책을 적용(NIST AU-9·AU-6)</t>
         </is>
       </c>
       <c r="AO22" s="9" t="inlineStr">
         <is>
-          <t>LOLDrivers 〈Project〉
-Hive Security 〈Modern Attack Techniques 2026〉</t>
+          <t>MITRE 〈ATT&amp;CK Enterprise v19.2〉</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[ST] 은닉</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-01.2</t>
+          <t>ENT-ST-02</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>보안 도구 무력화·드라이버 로드</t>
+          <t>위장(정상 이름·서명)</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>취약·악성 드라이버 로드(커널)</t>
+          <t>위장(정상 이름·경로·서명 가장)</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>취약·악성 드라이버 로드로 커널 은닉·무력화 토대 마련</t>
+          <t>정상 이름·경로·서명 가장(위장)으로 눈·규칙 탐지 회피</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>- 공격자는 취약·악성 드라이버를 커널에 올려 은닉·무력화의 토대를 만들 수 있음
-- 커널 계층이라 상위 보안 제품이 보지 못함</t>
+          <t>- 공격자는 정상 프로세스·경로·서명으로 위장해 사람 눈과 규칙 기반 탐지를 피할 수 있음
+- 정상처럼 보여 레거시가 구분하기 어려우나 단독 피해는 제한적임</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>Load vulnerable/malicious kernel driver</t>
+          <t>Masquerading</t>
         </is>
       </c>
       <c r="H23" s="9" t="inlineStr">
@@ -12504,44 +12535,40 @@
       </c>
       <c r="I23" s="9" t="inlineStr">
         <is>
-          <t>커널·펌웨어 하위 계층</t>
+          <t>서명된 정상 도구 악용 · 시그니처 회피</t>
         </is>
       </c>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t>행위·네트워크·아이덴티티</t>
+          <t>EDR·XDR</t>
         </is>
       </c>
       <c r="K23" s="9" t="inlineStr">
         <is>
-          <t>국가배후 · 랜섬웨어</t>
+          <t>국가배후 · 랜섬웨어 · 사이버범죄</t>
         </is>
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Windows</t>
+          <t>Windows · Linux · macOS</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>T1543.003</t>
+          <t>T1036</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>T1543.003 Create or Modify System Process: Windows Service</t>
+          <t>T1036 Masquerading</t>
         </is>
       </c>
       <c r="O23" s="8" t="n">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="P23" s="8" t="inlineStr"/>
       <c r="Q23" s="8" t="inlineStr"/>
-      <c r="R23" s="8" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
+      <c r="R23" s="8" t="inlineStr"/>
       <c r="S23" s="9" t="inlineStr"/>
       <c r="T23" s="9" t="inlineStr"/>
       <c r="U23" s="9" t="inlineStr"/>
@@ -12550,7 +12577,7 @@
       <c r="X23" s="9" t="inlineStr"/>
       <c r="Y23" s="8" t="inlineStr">
         <is>
-          <t>상</t>
+          <t>중</t>
         </is>
       </c>
       <c r="Z23" s="8" t="inlineStr">
@@ -12558,30 +12585,30 @@
           <t>중</t>
         </is>
       </c>
-      <c r="AA23" s="12" t="inlineStr">
-        <is>
-          <t>높음</t>
+      <c r="AA23" s="13" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="AB23" s="9" t="inlineStr"/>
       <c r="AC23" s="8" t="n">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="AD23" s="9" t="inlineStr">
         <is>
-          <t>실제 사고 3건(최근 2, 서로 다른 행위자·캠페인 3) · 빈발 지수 상(ATT&amp;CK 주체 140) · KEV - · 정부 경보 0 · 위협인텔 0 · 실증 0</t>
+          <t>실제 사고 0건(최근 0, 서로 다른 행위자·캠페인 0) · 빈발 지수 중(ATT&amp;CK 주체 60) · KEV - · 정부 경보 0 · 위협인텔 0 · 실증 0</t>
         </is>
       </c>
       <c r="AE23" s="9" t="inlineStr">
         <is>
-          <t>커널에 취약 드라이버를 올려 무력화·은닉의 토대를 만드는 단계 — 단독 피해는 없음</t>
+          <t>정상 프로세스·경로·서명으로 위장해 눈과 규칙 기반 탐지를 피하나 단독 피해는 제한적</t>
         </is>
       </c>
       <c r="AF23" s="9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AG23" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AH23" s="9" t="n">
         <v>0</v>
@@ -12589,78 +12616,68 @@
       <c r="AI23" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AJ23" s="27" t="inlineStr">
-        <is>
-          <t>실제 사고 확인</t>
-        </is>
-      </c>
-      <c r="AK23" s="9" t="inlineStr">
-        <is>
-          <t>ENI-016, ENI-017, ENI-036</t>
-        </is>
-      </c>
-      <c r="AL23" s="9" t="inlineStr">
-        <is>
-          <t>랜섬·암호화 2 · 자격증명·비밀 탈취 1 · 내부 접근 확보 1</t>
-        </is>
-      </c>
+      <c r="AJ23" s="28" t="inlineStr">
+        <is>
+          <t>ATT&amp;CK 사례·KEV 다수</t>
+        </is>
+      </c>
+      <c r="AK23" s="9" t="inlineStr"/>
+      <c r="AL23" s="9" t="inlineStr"/>
       <c r="AM23" s="9" t="inlineStr">
         <is>
-          <t>SI-7 Software, Firmware, and Information Integrity
-CM-7 Least Functionality
-SI-4 System Monitoring</t>
+          <t>SI-4 System Monitoring
+SI-7 Software, Firmware, and Information Integrity</t>
         </is>
       </c>
       <c r="AN23" s="9" t="inlineStr">
         <is>
           <t>■ 탐지
-- 신규 커널 드라이버 로드와 취약 드라이버 서명·해시를 차단 목록과 대조(NIST SI-7·SI-4)
+- 정상 이름과 다른 경로·서명·해시 불일치를 무결성·행위 기반으로 탐지(NIST SI-4·SI-7)
 ■ 대응
-- HVCI·드라이버 블록리스트로 취약 드라이버 로드를 차단(NIST SI-7·CM-7)
-- 참고: LOLDrivers 〈Project〉</t>
+- 바이너리 무결성·서명 검증과 정상 경로 기준선 대조를 적용(NIST SI-7·SI-4)</t>
         </is>
       </c>
       <c r="AO23" s="9" t="inlineStr">
         <is>
-          <t>LOLDrivers 〈Project〉</t>
+          <t>MITRE 〈ATT&amp;CK Enterprise v19.2〉</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[ST] 은닉</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-03</t>
+          <t>ENT-ST-03</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>지표 삭제</t>
+          <t>파일·정보 난독화</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>지표 삭제(이벤트 로그·파일 삭제)</t>
+          <t>파일·정보 난독화·암호화</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>이벤트 로그·파일 삭제로 레거시 SIEM 탐지·분석 무력화</t>
+          <t>패킹·인코딩·암호화 난독화로 시그니처·정적 분석 회피</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>- 공격자는 이벤트 로그·파일을 지워 레거시 SIEM 탐지와 사후 분석을 무력화할 수 있음
-- 원격·불변 로그가 없으면 흔적이 사라져 추적이 어려워짐</t>
+          <t>- 공격자는 페이로드를 패킹·인코딩·암호화해 시그니처·정적 분석을 회피할 수 있음
+- 변종 양산으로 레거시 AV를 지속 우회하나 단독 피해는 제한적임</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>Indicator removal (clear event logs, file deletion)</t>
+          <t>Obfuscated files or information</t>
         </is>
       </c>
       <c r="H24" s="9" t="inlineStr">
@@ -12670,38 +12687,36 @@
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>시그니처 회피</t>
+          <t>시그니처 회피 · 파일리스·인메모리</t>
         </is>
       </c>
       <c r="J24" s="8" t="inlineStr">
         <is>
-          <t>행위·네트워크·아이덴티티</t>
+          <t>EDR·XDR</t>
         </is>
       </c>
       <c r="K24" s="9" t="inlineStr">
         <is>
-          <t>국가배후 · 랜섬웨어</t>
+          <t>사이버범죄 · 랜섬웨어 · 국가배후</t>
         </is>
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Windows · Linux</t>
+          <t>Windows · Linux · macOS</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>T1070, T1070.004, T1685.005</t>
+          <t>T1027</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
         <is>
-          <t>T1070 Indicator Removal
-T1070.004 Indicator Removal: File Deletion
-T1685.005 Disable or Modify Tools: Clear Windows Event Logs</t>
+          <t>T1027 Obfuscated Files or Information</t>
         </is>
       </c>
       <c r="O24" s="8" t="n">
-        <v>335</v>
+        <v>160</v>
       </c>
       <c r="P24" s="8" t="inlineStr"/>
       <c r="Q24" s="8" t="inlineStr"/>
@@ -12714,7 +12729,7 @@
       <c r="X24" s="9" t="inlineStr"/>
       <c r="Y24" s="8" t="inlineStr">
         <is>
-          <t>상</t>
+          <t>중</t>
         </is>
       </c>
       <c r="Z24" s="8" t="inlineStr">
@@ -12722,30 +12737,30 @@
           <t>중</t>
         </is>
       </c>
-      <c r="AA24" s="12" t="inlineStr">
-        <is>
-          <t>높음</t>
+      <c r="AA24" s="13" t="inlineStr">
+        <is>
+          <t>보통</t>
         </is>
       </c>
       <c r="AB24" s="9" t="inlineStr"/>
       <c r="AC24" s="8" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="AD24" s="9" t="inlineStr">
         <is>
-          <t>실제 사고 2건(최근 1, 서로 다른 행위자·캠페인 2) · 빈발 지수 상(ATT&amp;CK 주체 335) · KEV - · 정부 경보 0 · 위협인텔 0 · 실증 0</t>
+          <t>실제 사고 0건(최근 0, 서로 다른 행위자·캠페인 0) · 빈발 지수 상(ATT&amp;CK 주체 160) · KEV - · 정부 경보 0 · 위협인텔 0 · 실증 0</t>
         </is>
       </c>
       <c r="AE24" s="9" t="inlineStr">
         <is>
-          <t>이벤트 로그·파일을 지워 레거시 SIEM 탐지·사후 분석을 무력화 — 원격·불변 로그가 없으면 흔적이 사라짐</t>
+          <t>패킹·인코딩·암호화로 시그니처·정적 분석을 회피 — 변종 양산으로 레거시 AV를 지속 우회</t>
         </is>
       </c>
       <c r="AF24" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AG24" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH24" s="9" t="n">
         <v>0</v>
@@ -12753,34 +12768,25 @@
       <c r="AI24" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AJ24" s="27" t="inlineStr">
-        <is>
-          <t>실제 사고 확인</t>
-        </is>
-      </c>
-      <c r="AK24" s="9" t="inlineStr">
-        <is>
-          <t>ENI-001, ENI-034</t>
-        </is>
-      </c>
-      <c r="AL24" s="9" t="inlineStr">
-        <is>
-          <t>내부 접근 확보 2 · 첩보·감시 1 · 측면 이동·확산 1 · 데이터 유출 1</t>
-        </is>
-      </c>
+      <c r="AJ24" s="28" t="inlineStr">
+        <is>
+          <t>ATT&amp;CK 사례·KEV 다수</t>
+        </is>
+      </c>
+      <c r="AK24" s="9" t="inlineStr"/>
+      <c r="AL24" s="9" t="inlineStr"/>
       <c r="AM24" s="9" t="inlineStr">
         <is>
-          <t>AU-9 Protection of Audit Information
-SI-4 System Monitoring
-AU-6 Audit Record Review, Analysis, and Reporting</t>
+          <t>SI-3 Malicious Code Protection
+SI-4 System Monitoring</t>
         </is>
       </c>
       <c r="AN24" s="9" t="inlineStr">
         <is>
           <t>■ 탐지
-- 로그 삭제·감사 정책 변경 이벤트와 원격 수집 로그의 공백을 모니터링(NIST AU-6·SI-4)
+- 실행 시점 행위·언패킹과 비정상 인코딩·엔트로피를 행위 기반으로 탐지(NIST SI-3·SI-4)
 ■ 대응
-- 원격·불변 로그 전송과 로그 삭제 방지·보존 정책을 적용(NIST AU-9·AU-6)</t>
+- 시그니처 의존을 줄이고 행위 기반·샌드박스 분석을 병행(NIST SI-3·SI-4)</t>
         </is>
       </c>
       <c r="AO24" s="9" t="inlineStr">
@@ -12792,38 +12798,38 @@
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[ST] 은닉</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-04</t>
+          <t>ENT-ST-04</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>위장(정상 이름·서명)</t>
+          <t>인메모리·반사 로딩</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>위장(정상 이름·경로·서명 가장)</t>
+          <t>인메모리·반사 코드 로딩</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>정상 이름·경로·서명 가장(위장)으로 눈·규칙 탐지 회피</t>
+          <t>인메모리·반사 코드 로딩으로 파일 기반 AV 원천 회피</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>- 공격자는 정상 프로세스·경로·서명으로 위장해 사람 눈과 규칙 기반 탐지를 피할 수 있음
-- 정상처럼 보여 레거시가 구분하기 어려우나 단독 피해는 제한적임</t>
+          <t>- 공격자는 디스크를 거치지 않고 메모리에서 페이로드를 로드·실행할 수 있음
+- 파일 기반 AV·시그니처가 원천적으로 보지 못해 행위·메모리 기반 탐지가 필요함</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>Masquerading</t>
+          <t>In-memory / reflective code loading</t>
         </is>
       </c>
       <c r="H25" s="9" t="inlineStr">
@@ -12833,36 +12839,36 @@
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>서명된 정상 도구 악용 · 시그니처 회피</t>
+          <t>파일리스·인메모리 · 시그니처 회피</t>
         </is>
       </c>
       <c r="J25" s="8" t="inlineStr">
         <is>
-          <t>EDR·XDR</t>
+          <t>행위·네트워크·아이덴티티</t>
         </is>
       </c>
       <c r="K25" s="9" t="inlineStr">
         <is>
-          <t>국가배후 · 랜섬웨어 · 사이버범죄</t>
+          <t>국가배후 · 랜섬웨어</t>
         </is>
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Windows · Linux · macOS</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>T1036</t>
+          <t>T1620</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>T1036 Masquerading</t>
+          <t>T1620 Reflective Code Loading</t>
         </is>
       </c>
       <c r="O25" s="8" t="n">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="P25" s="8" t="inlineStr"/>
       <c r="Q25" s="8" t="inlineStr"/>
@@ -12890,16 +12896,16 @@
       </c>
       <c r="AB25" s="9" t="inlineStr"/>
       <c r="AC25" s="8" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="AD25" s="9" t="inlineStr">
         <is>
-          <t>실제 사고 0건(최근 0, 서로 다른 행위자·캠페인 0) · 빈발 지수 중(ATT&amp;CK 주체 60) · KEV - · 정부 경보 0 · 위협인텔 0 · 실증 0</t>
+          <t>실제 사고 0건(최근 0, 서로 다른 행위자·캠페인 0) · 빈발 지수 중(ATT&amp;CK 주체 32) · KEV - · 정부 경보 0 · 위협인텔 0 · 실증 0</t>
         </is>
       </c>
       <c r="AE25" s="9" t="inlineStr">
         <is>
-          <t>정상 프로세스·경로·서명으로 위장해 눈과 규칙 기반 탐지를 피하나 단독 피해는 제한적</t>
+          <t>메모리 로딩으로 탐지를 회피하는 은닉 수단 — 단독 피해 없음</t>
         </is>
       </c>
       <c r="AF25" s="9" t="n">
@@ -12923,16 +12929,16 @@
       <c r="AL25" s="9" t="inlineStr"/>
       <c r="AM25" s="9" t="inlineStr">
         <is>
-          <t>SI-4 System Monitoring
-SI-7 Software, Firmware, and Information Integrity</t>
+          <t>SI-3 Malicious Code Protection
+SI-4 System Monitoring</t>
         </is>
       </c>
       <c r="AN25" s="9" t="inlineStr">
         <is>
           <t>■ 탐지
-- 정상 이름과 다른 경로·서명·해시 불일치를 무결성·행위 기반으로 탐지(NIST SI-4·SI-7)
+- 메모리 영역 할당·실행과 비정상 로딩을 EDR 메모리 스캔으로 탐지(NIST SI-3·SI-4)
 ■ 대응
-- 바이너리 무결성·서명 검증과 정상 경로 기준선 대조를 적용(NIST SI-7·SI-4)</t>
+- 메모리 가시성(EDR)·공격 표면 축소와 스크립트 실행 통제를 적용(NIST SI-3·SI-4)</t>
         </is>
       </c>
       <c r="AO25" s="9" t="inlineStr">
@@ -12944,38 +12950,38 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[ST] 은닉</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-05</t>
+          <t>ENT-ST-05</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>파일·정보 난독화</t>
+          <t>루트킷</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>파일·정보 난독화·암호화</t>
+          <t>루트킷(사용자·커널 은폐)</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>패킹·인코딩·암호화 난독화로 시그니처·정적 분석 회피</t>
+          <t>루트킷으로 프로세스·파일·연결을 하위 계층에서 은폐</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>- 공격자는 페이로드를 패킹·인코딩·암호화해 시그니처·정적 분석을 회피할 수 있음
-- 변종 양산으로 레거시 AV를 지속 우회하나 단독 피해는 제한적임</t>
+          <t>- 공격자는 루트킷으로 프로세스·파일·연결을 하위 계층에서 숨겨 탐지·분석을 방해할 수 있음
+- 레거시로는 존재 자체를 알기 어려워 장기 잠복에 쓰임</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>Obfuscated files or information</t>
+          <t>Rootkit</t>
         </is>
       </c>
       <c r="H26" s="9" t="inlineStr">
@@ -12985,36 +12991,36 @@
       </c>
       <c r="I26" s="9" t="inlineStr">
         <is>
-          <t>시그니처 회피 · 파일리스·인메모리</t>
+          <t>커널·펌웨어 하위 계층 · 파일리스·인메모리</t>
         </is>
       </c>
       <c r="J26" s="8" t="inlineStr">
         <is>
-          <t>EDR·XDR</t>
+          <t>행위·네트워크·아이덴티티</t>
         </is>
       </c>
       <c r="K26" s="9" t="inlineStr">
         <is>
-          <t>사이버범죄 · 랜섬웨어 · 국가배후</t>
+          <t>국가배후</t>
         </is>
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Windows · Linux · macOS</t>
+          <t>Windows · Linux</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>T1027</t>
+          <t>T1014</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>T1027 Obfuscated Files or Information</t>
+          <t>T1014 Rootkit</t>
         </is>
       </c>
       <c r="O26" s="8" t="n">
-        <v>160</v>
+        <v>32</v>
       </c>
       <c r="P26" s="8" t="inlineStr"/>
       <c r="Q26" s="8" t="inlineStr"/>
@@ -13042,16 +13048,16 @@
       </c>
       <c r="AB26" s="9" t="inlineStr"/>
       <c r="AC26" s="8" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="AD26" s="9" t="inlineStr">
         <is>
-          <t>실제 사고 0건(최근 0, 서로 다른 행위자·캠페인 0) · 빈발 지수 상(ATT&amp;CK 주체 160) · KEV - · 정부 경보 0 · 위협인텔 0 · 실증 0</t>
+          <t>실제 사고 0건(최근 0, 서로 다른 행위자·캠페인 0) · 빈발 지수 중(ATT&amp;CK 주체 32) · KEV - · 정부 경보 0 · 위협인텔 0 · 실증 0</t>
         </is>
       </c>
       <c r="AE26" s="9" t="inlineStr">
         <is>
-          <t>패킹·인코딩·암호화로 시그니처·정적 분석을 회피 — 변종 양산으로 레거시 AV를 지속 우회</t>
+          <t>루트킷으로 존재를 은폐해 장기 잠복하는 은닉 수단 — 직접 피해보다 지속·은닉 조건</t>
         </is>
       </c>
       <c r="AF26" s="9" t="n">
@@ -13075,16 +13081,16 @@
       <c r="AL26" s="9" t="inlineStr"/>
       <c r="AM26" s="9" t="inlineStr">
         <is>
-          <t>SI-3 Malicious Code Protection
+          <t>SI-7 Software, Firmware, and Information Integrity
 SI-4 System Monitoring</t>
         </is>
       </c>
       <c r="AN26" s="9" t="inlineStr">
         <is>
           <t>■ 탐지
-- 실행 시점 행위·언패킹과 비정상 인코딩·엔트로피를 행위 기반으로 탐지(NIST SI-3·SI-4)
+- 커널 무결성·드라이버 서명과 메모리·부트 무결성 검증으로 은폐를 탐지(NIST SI-7·SI-4)
 ■ 대응
-- 시그니처 의존을 줄이고 행위 기반·샌드박스 분석을 병행(NIST SI-3·SI-4)</t>
+- 커널 무결성 보호(HVCI)·보안 부팅과 하위 계층 텔레메트리를 확보(NIST SI-7·SI-4)</t>
         </is>
       </c>
       <c r="AO26" s="9" t="inlineStr">
@@ -13096,38 +13102,38 @@
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[ST] 은닉</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-06</t>
+          <t>ENT-ST-06</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>인메모리·반사 로딩</t>
+          <t>펌웨어·부트 수준 은닉</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>인메모리·반사 코드 로딩</t>
+          <t>펌웨어·부트킷(UEFI) 지속·은닉</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>인메모리·반사 코드 로딩으로 파일 기반 AV 원천 회피</t>
+          <t>펌웨어·부트킷(UEFI)으로 OS 아래 지속·은닉</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>- 공격자는 디스크를 거치지 않고 메모리에서 페이로드를 로드·실행할 수 있음
-- 파일 기반 AV·시그니처가 원천적으로 보지 못해 행위·메모리 기반 탐지가 필요함</t>
+          <t>- 공격자는 OS 아래 펌웨어·부트 단계에 임플란트를 심어 재설치·디스크 교체에도 지속할 수 있음
+- OS 보안 제품의 가시성 밖이라 레거시·EDR 모두 사실상 공백임</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>In-memory / reflective code loading</t>
+          <t>Pre-OS boot / firmware implant (bootkit)</t>
         </is>
       </c>
       <c r="H27" s="9" t="inlineStr">
@@ -13137,7 +13143,7 @@
       </c>
       <c r="I27" s="9" t="inlineStr">
         <is>
-          <t>파일리스·인메모리 · 시그니처 회피</t>
+          <t>커널·펌웨어 하위 계층</t>
         </is>
       </c>
       <c r="J27" s="8" t="inlineStr">
@@ -13147,26 +13153,26 @@
       </c>
       <c r="K27" s="9" t="inlineStr">
         <is>
-          <t>국가배후 · 랜섬웨어</t>
+          <t>국가배후</t>
         </is>
       </c>
       <c r="L27" s="9" t="inlineStr">
         <is>
-          <t>Windows</t>
+          <t>펌웨어 · Windows</t>
         </is>
       </c>
       <c r="M27" s="9" t="inlineStr">
         <is>
-          <t>T1620</t>
+          <t>T1542</t>
         </is>
       </c>
       <c r="N27" s="9" t="inlineStr">
         <is>
-          <t>T1620 Reflective Code Loading</t>
+          <t>T1542 Pre-OS Boot</t>
         </is>
       </c>
       <c r="O27" s="8" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="P27" s="8" t="inlineStr"/>
       <c r="Q27" s="8" t="inlineStr"/>
@@ -13194,20 +13200,20 @@
       </c>
       <c r="AB27" s="9" t="inlineStr"/>
       <c r="AC27" s="8" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="AD27" s="9" t="inlineStr">
         <is>
-          <t>실제 사고 0건(최근 0, 서로 다른 행위자·캠페인 0) · 빈발 지수 중(ATT&amp;CK 주체 32) · KEV - · 정부 경보 0 · 위협인텔 0 · 실증 0</t>
+          <t>실제 사고 1건(최근 0, 서로 다른 행위자·캠페인 1) · 빈발 지수 하(ATT&amp;CK 주체 0) · KEV - · 정부 경보 0 · 위협인텔 0 · 실증 1</t>
         </is>
       </c>
       <c r="AE27" s="9" t="inlineStr">
         <is>
-          <t>메모리 로딩으로 탐지를 회피하는 은닉 수단 — 단독 피해 없음</t>
+          <t>펌웨어·부트킷으로 재설치에도 지속하는 하위 계층 지속성 — 직접 피해보다 장기 지속 조건</t>
         </is>
       </c>
       <c r="AF27" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG27" s="9" t="n">
         <v>0</v>
@@ -13218,25 +13224,34 @@
       <c r="AI27" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AJ27" s="28" t="inlineStr">
-        <is>
-          <t>ATT&amp;CK 사례·KEV 다수</t>
-        </is>
-      </c>
-      <c r="AK27" s="9" t="inlineStr"/>
-      <c r="AL27" s="9" t="inlineStr"/>
+      <c r="AJ27" s="27" t="inlineStr">
+        <is>
+          <t>실제 사고 확인</t>
+        </is>
+      </c>
+      <c r="AK27" s="9" t="inlineStr">
+        <is>
+          <t>ENI-026
+실증: ENI-024</t>
+        </is>
+      </c>
+      <c r="AL27" s="9" t="inlineStr">
+        <is>
+          <t>내부 접근 확보 1 · 첩보·감시 1</t>
+        </is>
+      </c>
       <c r="AM27" s="9" t="inlineStr">
         <is>
-          <t>SI-3 Malicious Code Protection
-SI-4 System Monitoring</t>
+          <t>SI-7 Software, Firmware, and Information Integrity
+CM-7 Least Functionality</t>
         </is>
       </c>
       <c r="AN27" s="9" t="inlineStr">
         <is>
           <t>■ 탐지
-- 메모리 영역 할당·실행과 비정상 로딩을 EDR 메모리 스캔으로 탐지(NIST SI-3·SI-4)
+- 펌웨어·부트 무결성 측정(보안 부팅·측정 부팅)과 펌웨어 버전·해시 변화를 점검(NIST SI-7)
 ■ 대응
-- 메모리 가시성(EDR)·공격 표면 축소와 스크립트 실행 통제를 적용(NIST SI-3·SI-4)</t>
+- 보안 부팅·펌웨어 무결성 검증·업데이트와 펌웨어 공급 신뢰를 관리(NIST SI-7·CM-7)</t>
         </is>
       </c>
       <c r="AO27" s="9" t="inlineStr">
@@ -13248,38 +13263,38 @@
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[DM] 방어 무력화</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-07</t>
+          <t>ENT-DM-01.1</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>루트킷</t>
+          <t>보안 도구 무력화·드라이버 로드</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>루트킷(사용자·커널 은폐)</t>
+          <t>보안 도구 무력화(EDR 변조·BYOVD EDR 킬러)</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>루트킷으로 프로세스·파일·연결을 하위 계층에서 은폐</t>
+          <t>서명된 취약 드라이버로 EDR·백신을 커널에서 무력화(BYOVD)</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>- 공격자는 루트킷으로 프로세스·파일·연결을 하위 계층에서 숨겨 탐지·분석을 방해할 수 있음
-- 레거시로는 존재 자체를 알기 어려워 장기 잠복에 쓰임</t>
+          <t>- 공격자는 서명된 취약 드라이버를 올려 EDR·백신을 커널에서 무력화할 수 있음
+- 보안 도구 자체가 꺼지므로 이후 단계가 전부 가려지고, 여러 랜섬웨어·국가배후가 EDR 킬러를 공유함</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>Rootkit</t>
+          <t>Impair/disable security tools (EDR tampering, BYOVD killers)</t>
         </is>
       </c>
       <c r="H28" s="9" t="inlineStr">
@@ -13289,7 +13304,7 @@
       </c>
       <c r="I28" s="9" t="inlineStr">
         <is>
-          <t>커널·펌웨어 하위 계층 · 파일리스·인메모리</t>
+          <t>커널·펌웨어 하위 계층 · 서명된 정상 도구 악용</t>
         </is>
       </c>
       <c r="J28" s="8" t="inlineStr">
@@ -13299,30 +13314,34 @@
       </c>
       <c r="K28" s="9" t="inlineStr">
         <is>
-          <t>국가배후</t>
+          <t>랜섬웨어 · 국가배후</t>
         </is>
       </c>
       <c r="L28" s="9" t="inlineStr">
         <is>
-          <t>Windows · Linux</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>T1014</t>
+          <t>T1685</t>
         </is>
       </c>
       <c r="N28" s="9" t="inlineStr">
         <is>
-          <t>T1014 Rootkit</t>
+          <t>T1685 Disable or Modify Tools</t>
         </is>
       </c>
       <c r="O28" s="8" t="n">
-        <v>32</v>
+        <v>155</v>
       </c>
       <c r="P28" s="8" t="inlineStr"/>
       <c r="Q28" s="8" t="inlineStr"/>
-      <c r="R28" s="8" t="inlineStr"/>
+      <c r="R28" s="8" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="S28" s="9" t="inlineStr"/>
       <c r="T28" s="9" t="inlineStr"/>
       <c r="U28" s="9" t="inlineStr"/>
@@ -13331,107 +13350,119 @@
       <c r="X28" s="9" t="inlineStr"/>
       <c r="Y28" s="8" t="inlineStr">
         <is>
+          <t>상</t>
+        </is>
+      </c>
+      <c r="Z28" s="8" t="inlineStr">
+        <is>
           <t>중</t>
         </is>
       </c>
-      <c r="Z28" s="8" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="AA28" s="13" t="inlineStr">
-        <is>
-          <t>보통</t>
+      <c r="AA28" s="12" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
       <c r="AB28" s="9" t="inlineStr"/>
       <c r="AC28" s="8" t="n">
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="AD28" s="9" t="inlineStr">
         <is>
-          <t>실제 사고 0건(최근 0, 서로 다른 행위자·캠페인 0) · 빈발 지수 중(ATT&amp;CK 주체 32) · KEV - · 정부 경보 0 · 위협인텔 0 · 실증 0</t>
+          <t>실제 사고 7건(최근 3, 서로 다른 행위자·캠페인 7) · 빈발 지수 상(ATT&amp;CK 주체 155) · KEV - · 정부 경보 1 · 위협인텔 0 · 실증 0</t>
         </is>
       </c>
       <c r="AE28" s="9" t="inlineStr">
         <is>
-          <t>루트킷으로 존재를 은폐해 장기 잠복하는 은닉 수단 — 직접 피해보다 지속·은닉 조건</t>
+          <t>EDR·백신을 무력화해 이후 단계를 가리는 방어 무력화 수단 — 단독 피해보다 공격 성공률을 높이는 조건</t>
         </is>
       </c>
       <c r="AF28" s="9" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AG28" s="9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AH28" s="9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI28" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="AJ28" s="28" t="inlineStr">
-        <is>
-          <t>ATT&amp;CK 사례·KEV 다수</t>
-        </is>
-      </c>
-      <c r="AK28" s="9" t="inlineStr"/>
-      <c r="AL28" s="9" t="inlineStr"/>
+      <c r="AJ28" s="27" t="inlineStr">
+        <is>
+          <t>실제 사고 확인</t>
+        </is>
+      </c>
+      <c r="AK28" s="9" t="inlineStr">
+        <is>
+          <t>ENI-012, ENI-013, ENI-015, ENI-016, ENI-017, ENI-036, ENI-037
+정부 경보: ENI-030</t>
+        </is>
+      </c>
+      <c r="AL28" s="9" t="inlineStr">
+        <is>
+          <t>랜섬·암호화 6 · 데이터 유출 2 · 자격증명·비밀 탈취 2 · 내부 접근 확보 2</t>
+        </is>
+      </c>
       <c r="AM28" s="9" t="inlineStr">
         <is>
-          <t>SI-7 Software, Firmware, and Information Integrity
-SI-4 System Monitoring</t>
+          <t>SI-4 System Monitoring
+SI-7 Software, Firmware, and Information Integrity
+CM-7 Least Functionality</t>
         </is>
       </c>
       <c r="AN28" s="9" t="inlineStr">
         <is>
           <t>■ 탐지
-- 커널 무결성·드라이버 서명과 메모리·부트 무결성 검증으로 은폐를 탐지(NIST SI-7·SI-4)
+- 보안 서비스 중지·드라이버 로드와 EDR 텔레메트리 단절을 행위·네트워크 기반으로 탐지(NIST SI-4·SI-7)
 ■ 대응
-- 커널 무결성 보호(HVCI)·보안 부팅과 하위 계층 텔레메트리를 확보(NIST SI-7·SI-4)</t>
+- 취약 드라이버 차단 목록(HVCI·블록리스트)·변조 방지와 보안 도구 상태를 중앙 감시(NIST SI-7·CM-7)
+- 참고: LOLDrivers 〈Project〉 · Hive Security 〈Modern Attack Techniques 2026〉</t>
         </is>
       </c>
       <c r="AO28" s="9" t="inlineStr">
         <is>
-          <t>MITRE 〈ATT&amp;CK Enterprise v19.2〉</t>
+          <t>LOLDrivers 〈Project〉
+Hive Security 〈Modern Attack Techniques 2026〉</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[DM] 방어 무력화</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-08</t>
+          <t>ENT-DM-01.2</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>펌웨어·부트 수준 은닉</t>
+          <t>보안 도구 무력화·드라이버 로드</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>펌웨어·부트킷(UEFI) 지속·은닉</t>
+          <t>취약·악성 드라이버 로드(커널)</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>펌웨어·부트킷(UEFI)으로 OS 아래 지속·은닉</t>
+          <t>취약·악성 드라이버 로드로 커널 은닉·무력화 토대 마련</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>- 공격자는 OS 아래 펌웨어·부트 단계에 임플란트를 심어 재설치·디스크 교체에도 지속할 수 있음
-- OS 보안 제품의 가시성 밖이라 레거시·EDR 모두 사실상 공백임</t>
+          <t>- 공격자는 취약·악성 드라이버를 커널에 올려 은닉·무력화의 토대를 만들 수 있음
+- 커널 계층이라 상위 보안 제품이 보지 못함</t>
         </is>
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>Pre-OS boot / firmware implant (bootkit)</t>
+          <t>Load vulnerable/malicious kernel driver</t>
         </is>
       </c>
       <c r="H29" s="9" t="inlineStr">
@@ -13451,30 +13482,34 @@
       </c>
       <c r="K29" s="9" t="inlineStr">
         <is>
-          <t>국가배후</t>
+          <t>국가배후 · 랜섬웨어</t>
         </is>
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>펌웨어 · Windows</t>
+          <t>Windows</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>T1542</t>
+          <t>T1543.003</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>T1542 Pre-OS Boot</t>
+          <t>T1543.003 Create or Modify System Process: Windows Service</t>
         </is>
       </c>
       <c r="O29" s="8" t="n">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="P29" s="8" t="inlineStr"/>
       <c r="Q29" s="8" t="inlineStr"/>
-      <c r="R29" s="8" t="inlineStr"/>
+      <c r="R29" s="8" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
       <c r="S29" s="9" t="inlineStr"/>
       <c r="T29" s="9" t="inlineStr"/>
       <c r="U29" s="9" t="inlineStr"/>
@@ -13483,38 +13518,38 @@
       <c r="X29" s="9" t="inlineStr"/>
       <c r="Y29" s="8" t="inlineStr">
         <is>
+          <t>상</t>
+        </is>
+      </c>
+      <c r="Z29" s="8" t="inlineStr">
+        <is>
           <t>중</t>
         </is>
       </c>
-      <c r="Z29" s="8" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="AA29" s="13" t="inlineStr">
-        <is>
-          <t>보통</t>
+      <c r="AA29" s="12" t="inlineStr">
+        <is>
+          <t>높음</t>
         </is>
       </c>
       <c r="AB29" s="9" t="inlineStr"/>
       <c r="AC29" s="8" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="AD29" s="9" t="inlineStr">
         <is>
-          <t>실제 사고 1건(최근 0, 서로 다른 행위자·캠페인 1) · 빈발 지수 하(ATT&amp;CK 주체 0) · KEV - · 정부 경보 0 · 위협인텔 0 · 실증 1</t>
+          <t>실제 사고 3건(최근 2, 서로 다른 행위자·캠페인 3) · 빈발 지수 상(ATT&amp;CK 주체 140) · KEV - · 정부 경보 0 · 위협인텔 0 · 실증 0</t>
         </is>
       </c>
       <c r="AE29" s="9" t="inlineStr">
         <is>
-          <t>펌웨어·부트킷으로 재설치에도 지속하는 하위 계층 지속성 — 직접 피해보다 장기 지속 조건</t>
+          <t>커널에 취약 드라이버를 올려 무력화·은닉의 토대를 만드는 단계 — 단독 피해는 없음</t>
         </is>
       </c>
       <c r="AF29" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AG29" s="9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AH29" s="9" t="n">
         <v>0</v>
@@ -13529,32 +13564,33 @@
       </c>
       <c r="AK29" s="9" t="inlineStr">
         <is>
-          <t>ENI-026
-실증: ENI-024</t>
+          <t>ENI-016, ENI-017, ENI-036</t>
         </is>
       </c>
       <c r="AL29" s="9" t="inlineStr">
         <is>
-          <t>내부 접근 확보 1 · 첩보·감시 1</t>
+          <t>랜섬·암호화 2 · 자격증명·비밀 탈취 1 · 내부 접근 확보 1</t>
         </is>
       </c>
       <c r="AM29" s="9" t="inlineStr">
         <is>
           <t>SI-7 Software, Firmware, and Information Integrity
-CM-7 Least Functionality</t>
+CM-7 Least Functionality
+SI-4 System Monitoring</t>
         </is>
       </c>
       <c r="AN29" s="9" t="inlineStr">
         <is>
           <t>■ 탐지
-- 펌웨어·부트 무결성 측정(보안 부팅·측정 부팅)과 펌웨어 버전·해시 변화를 점검(NIST SI-7)
+- 신규 커널 드라이버 로드와 취약 드라이버 서명·해시를 차단 목록과 대조(NIST SI-7·SI-4)
 ■ 대응
-- 보안 부팅·펌웨어 무결성 검증·업데이트와 펌웨어 공급 신뢰를 관리(NIST SI-7·CM-7)</t>
+- HVCI·드라이버 블록리스트로 취약 드라이버 로드를 차단(NIST SI-7·CM-7)
+- 참고: LOLDrivers 〈Project〉</t>
         </is>
       </c>
       <c r="AO29" s="9" t="inlineStr">
         <is>
-          <t>MITRE 〈ATT&amp;CK Enterprise v19.2〉</t>
+          <t>LOLDrivers 〈Project〉</t>
         </is>
       </c>
     </row>
@@ -14552,7 +14588,7 @@
       <c r="F36" s="9" t="inlineStr">
         <is>
           <t>- 공격자는 설치된 보안 제품을 확인해 회피·무력화를 준비할 수 있음
-- 사전 단계라 직접 피해는 없으나 이후 방어 회피로 이어짐</t>
+- 사전 단계라 직접 피해는 없으나 이후 은닉·방어 무력화로 이어짐</t>
         </is>
       </c>
       <c r="G36" s="9" t="inlineStr">
@@ -19407,81 +19443,597 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[ST] 은닉</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-01.1</t>
+          <t>ENT-ST-01</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
+          <t>지표 삭제</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>지표 삭제(이벤트 로그·파일 삭제)</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>이벤트 로그·파일 삭제로 레거시 SIEM 탐지·분석 무력화</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>- 공격자는 이벤트 로그·파일을 지워 레거시 SIEM 탐지와 사후 분석을 무력화할 수 있음
+- 원격·불변 로그가 없으면 흔적이 사라져 추적이 어려워짐</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>시그니처 회피</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>행위·네트워크·아이덴티티</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>Windows · Linux</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>상</t>
+        </is>
+      </c>
+      <c r="K20" s="8" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="L20" s="12" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="M20" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="N20" s="27" t="inlineStr">
+        <is>
+          <t>실제 사고 확인</t>
+        </is>
+      </c>
+      <c r="O20" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="P20" s="8" t="n">
+        <v>335</v>
+      </c>
+      <c r="Q20" s="8" t="inlineStr"/>
+      <c r="R20" s="9" t="inlineStr">
+        <is>
+          <t>■ 탐지
+- 로그 삭제·감사 정책 변경 이벤트와 원격 수집 로그의 공백을 모니터링(NIST AU-6·SI-4)
+■ 대응
+- 원격·불변 로그 전송과 로그 삭제 방지·보존 정책을 적용(NIST AU-9·AU-6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>[ST] 은닉</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>ENT-ST-02</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>위장(정상 이름·서명)</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>위장(정상 이름·경로·서명 가장)</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>정상 이름·경로·서명 가장(위장)으로 눈·규칙 탐지 회피</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>- 공격자는 정상 프로세스·경로·서명으로 위장해 사람 눈과 규칙 기반 탐지를 피할 수 있음
+- 정상처럼 보여 레거시가 구분하기 어려우나 단독 피해는 제한적임</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>서명된 정상 도구 악용 · 시그니처 회피</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>EDR·XDR</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>Windows · Linux · macOS</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="K21" s="8" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="L21" s="13" t="inlineStr">
+        <is>
+          <t>보통</t>
+        </is>
+      </c>
+      <c r="M21" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="N21" s="28" t="inlineStr">
+        <is>
+          <t>ATT&amp;CK 사례·KEV 다수</t>
+        </is>
+      </c>
+      <c r="O21" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q21" s="8" t="inlineStr"/>
+      <c r="R21" s="9" t="inlineStr">
+        <is>
+          <t>■ 탐지
+- 정상 이름과 다른 경로·서명·해시 불일치를 무결성·행위 기반으로 탐지(NIST SI-4·SI-7)
+■ 대응
+- 바이너리 무결성·서명 검증과 정상 경로 기준선 대조를 적용(NIST SI-7·SI-4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>[ST] 은닉</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>ENT-ST-03</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>파일·정보 난독화</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>파일·정보 난독화·암호화</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>패킹·인코딩·암호화 난독화로 시그니처·정적 분석 회피</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>- 공격자는 페이로드를 패킹·인코딩·암호화해 시그니처·정적 분석을 회피할 수 있음
+- 변종 양산으로 레거시 AV를 지속 우회하나 단독 피해는 제한적임</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>시그니처 회피 · 파일리스·인메모리</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>EDR·XDR</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Windows · Linux · macOS</t>
+        </is>
+      </c>
+      <c r="J22" s="8" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="K22" s="8" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="L22" s="13" t="inlineStr">
+        <is>
+          <t>보통</t>
+        </is>
+      </c>
+      <c r="M22" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="N22" s="28" t="inlineStr">
+        <is>
+          <t>ATT&amp;CK 사례·KEV 다수</t>
+        </is>
+      </c>
+      <c r="O22" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="8" t="n">
+        <v>160</v>
+      </c>
+      <c r="Q22" s="8" t="inlineStr"/>
+      <c r="R22" s="9" t="inlineStr">
+        <is>
+          <t>■ 탐지
+- 실행 시점 행위·언패킹과 비정상 인코딩·엔트로피를 행위 기반으로 탐지(NIST SI-3·SI-4)
+■ 대응
+- 시그니처 의존을 줄이고 행위 기반·샌드박스 분석을 병행(NIST SI-3·SI-4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>[ST] 은닉</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>ENT-ST-04</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>인메모리·반사 로딩</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>인메모리·반사 코드 로딩</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>인메모리·반사 코드 로딩으로 파일 기반 AV 원천 회피</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>- 공격자는 디스크를 거치지 않고 메모리에서 페이로드를 로드·실행할 수 있음
+- 파일 기반 AV·시그니처가 원천적으로 보지 못해 행위·메모리 기반 탐지가 필요함</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>파일리스·인메모리 · 시그니처 회피</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>행위·네트워크·아이덴티티</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="K23" s="8" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="L23" s="13" t="inlineStr">
+        <is>
+          <t>보통</t>
+        </is>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="N23" s="28" t="inlineStr">
+        <is>
+          <t>ATT&amp;CK 사례·KEV 다수</t>
+        </is>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="Q23" s="8" t="inlineStr"/>
+      <c r="R23" s="9" t="inlineStr">
+        <is>
+          <t>■ 탐지
+- 메모리 영역 할당·실행과 비정상 로딩을 EDR 메모리 스캔으로 탐지(NIST SI-3·SI-4)
+■ 대응
+- 메모리 가시성(EDR)·공격 표면 축소와 스크립트 실행 통제를 적용(NIST SI-3·SI-4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>[ST] 은닉</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>ENT-ST-05</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>루트킷</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>루트킷(사용자·커널 은폐)</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>루트킷으로 프로세스·파일·연결을 하위 계층에서 은폐</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>- 공격자는 루트킷으로 프로세스·파일·연결을 하위 계층에서 숨겨 탐지·분석을 방해할 수 있음
+- 레거시로는 존재 자체를 알기 어려워 장기 잠복에 쓰임</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>커널·펌웨어 하위 계층 · 파일리스·인메모리</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>행위·네트워크·아이덴티티</t>
+        </is>
+      </c>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>Windows · Linux</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="L24" s="13" t="inlineStr">
+        <is>
+          <t>보통</t>
+        </is>
+      </c>
+      <c r="M24" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="N24" s="28" t="inlineStr">
+        <is>
+          <t>ATT&amp;CK 사례·KEV 다수</t>
+        </is>
+      </c>
+      <c r="O24" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="Q24" s="8" t="inlineStr"/>
+      <c r="R24" s="9" t="inlineStr">
+        <is>
+          <t>■ 탐지
+- 커널 무결성·드라이버 서명과 메모리·부트 무결성 검증으로 은폐를 탐지(NIST SI-7·SI-4)
+■ 대응
+- 커널 무결성 보호(HVCI)·보안 부팅과 하위 계층 텔레메트리를 확보(NIST SI-7·SI-4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>[ST] 은닉</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>ENT-ST-06</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>펌웨어·부트 수준 은닉</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>펌웨어·부트킷(UEFI) 지속·은닉</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>펌웨어·부트킷(UEFI)으로 OS 아래 지속·은닉</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>- 공격자는 OS 아래 펌웨어·부트 단계에 임플란트를 심어 재설치·디스크 교체에도 지속할 수 있음
+- OS 보안 제품의 가시성 밖이라 레거시·EDR 모두 사실상 공백임</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>커널·펌웨어 하위 계층</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>행위·네트워크·아이덴티티</t>
+        </is>
+      </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>펌웨어 · Windows</t>
+        </is>
+      </c>
+      <c r="J25" s="8" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="K25" s="8" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t>보통</t>
+        </is>
+      </c>
+      <c r="M25" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="N25" s="27" t="inlineStr">
+        <is>
+          <t>실제 사고 확인</t>
+        </is>
+      </c>
+      <c r="O25" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P25" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="8" t="inlineStr"/>
+      <c r="R25" s="9" t="inlineStr">
+        <is>
+          <t>■ 탐지
+- 펌웨어·부트 무결성 측정(보안 부팅·측정 부팅)과 펌웨어 버전·해시 변화를 점검(NIST SI-7)
+■ 대응
+- 보안 부팅·펌웨어 무결성 검증·업데이트와 펌웨어 공급 신뢰를 관리(NIST SI-7·CM-7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>[DM] 방어 무력화</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>ENT-DM-01.1</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
           <t>보안 도구 무력화·드라이버 로드</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t>보안 도구 무력화(EDR 변조·BYOVD EDR 킬러)</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E26" s="9" t="inlineStr">
         <is>
           <t>서명된 취약 드라이버로 EDR·백신을 커널에서 무력화(BYOVD)</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>- 공격자는 서명된 취약 드라이버를 올려 EDR·백신을 커널에서 무력화할 수 있음
 - 보안 도구 자체가 꺼지므로 이후 단계가 전부 가려지고, 여러 랜섬웨어·국가배후가 EDR 킬러를 공유함</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G26" s="9" t="inlineStr">
         <is>
           <t>커널·펌웨어 하위 계층 · 서명된 정상 도구 악용</t>
         </is>
       </c>
-      <c r="H20" s="8" t="inlineStr">
+      <c r="H26" s="8" t="inlineStr">
         <is>
           <t>행위·네트워크·아이덴티티</t>
         </is>
       </c>
-      <c r="I20" s="9" t="inlineStr">
+      <c r="I26" s="9" t="inlineStr">
         <is>
           <t>Windows</t>
         </is>
       </c>
-      <c r="J20" s="8" t="inlineStr">
+      <c r="J26" s="8" t="inlineStr">
         <is>
           <t>상</t>
         </is>
       </c>
-      <c r="K20" s="8" t="inlineStr">
+      <c r="K26" s="8" t="inlineStr">
         <is>
           <t>중</t>
         </is>
       </c>
-      <c r="L20" s="12" t="inlineStr">
+      <c r="L26" s="12" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
       </c>
-      <c r="M20" s="8" t="n">
+      <c r="M26" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="N20" s="27" t="inlineStr">
+      <c r="N26" s="27" t="inlineStr">
         <is>
           <t>실제 사고 확인</t>
         </is>
       </c>
-      <c r="O20" s="8" t="n">
+      <c r="O26" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="P20" s="8" t="n">
+      <c r="P26" s="8" t="n">
         <v>155</v>
       </c>
-      <c r="Q20" s="8" t="inlineStr"/>
-      <c r="R20" s="9" t="inlineStr">
+      <c r="Q26" s="8" t="inlineStr"/>
+      <c r="R26" s="9" t="inlineStr">
         <is>
           <t>■ 탐지
 - 보안 서비스 중지·드라이버 로드와 EDR 텔레메트리 단절을 행위·네트워크 기반으로 탐지(NIST SI-4·SI-7)
@@ -19491,84 +20043,84 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>[DE] 방어 회피</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>ENT-DE-01.2</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>[DM] 방어 무력화</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>ENT-DM-01.2</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>보안 도구 무력화·드라이버 로드</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>취약·악성 드라이버 로드(커널)</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E27" s="9" t="inlineStr">
         <is>
           <t>취약·악성 드라이버 로드로 커널 은닉·무력화 토대 마련</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>- 공격자는 취약·악성 드라이버를 커널에 올려 은닉·무력화의 토대를 만들 수 있음
 - 커널 계층이라 상위 보안 제품이 보지 못함</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="G27" s="9" t="inlineStr">
         <is>
           <t>커널·펌웨어 하위 계층</t>
         </is>
       </c>
-      <c r="H21" s="8" t="inlineStr">
+      <c r="H27" s="8" t="inlineStr">
         <is>
           <t>행위·네트워크·아이덴티티</t>
         </is>
       </c>
-      <c r="I21" s="9" t="inlineStr">
+      <c r="I27" s="9" t="inlineStr">
         <is>
           <t>Windows</t>
         </is>
       </c>
-      <c r="J21" s="8" t="inlineStr">
+      <c r="J27" s="8" t="inlineStr">
         <is>
           <t>상</t>
         </is>
       </c>
-      <c r="K21" s="8" t="inlineStr">
+      <c r="K27" s="8" t="inlineStr">
         <is>
           <t>중</t>
         </is>
       </c>
-      <c r="L21" s="12" t="inlineStr">
+      <c r="L27" s="12" t="inlineStr">
         <is>
           <t>높음</t>
         </is>
       </c>
-      <c r="M21" s="8" t="n">
+      <c r="M27" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="N21" s="27" t="inlineStr">
+      <c r="N27" s="27" t="inlineStr">
         <is>
           <t>실제 사고 확인</t>
         </is>
       </c>
-      <c r="O21" s="8" t="n">
+      <c r="O27" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="P21" s="8" t="n">
+      <c r="P27" s="8" t="n">
         <v>140</v>
       </c>
-      <c r="Q21" s="8" t="inlineStr"/>
-      <c r="R21" s="9" t="inlineStr">
+      <c r="Q27" s="8" t="inlineStr"/>
+      <c r="R27" s="9" t="inlineStr">
         <is>
           <t>■ 탐지
 - 신규 커널 드라이버 로드와 취약 드라이버 서명·해시를 차단 목록과 대조(NIST SI-7·SI-4)
@@ -19578,522 +20130,6 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>[DE] 방어 회피</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>ENT-DE-03</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>지표 삭제</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>지표 삭제(이벤트 로그·파일 삭제)</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr">
-        <is>
-          <t>이벤트 로그·파일 삭제로 레거시 SIEM 탐지·분석 무력화</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>- 공격자는 이벤트 로그·파일을 지워 레거시 SIEM 탐지와 사후 분석을 무력화할 수 있음
-- 원격·불변 로그가 없으면 흔적이 사라져 추적이 어려워짐</t>
-        </is>
-      </c>
-      <c r="G22" s="9" t="inlineStr">
-        <is>
-          <t>시그니처 회피</t>
-        </is>
-      </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>행위·네트워크·아이덴티티</t>
-        </is>
-      </c>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>Windows · Linux</t>
-        </is>
-      </c>
-      <c r="J22" s="8" t="inlineStr">
-        <is>
-          <t>상</t>
-        </is>
-      </c>
-      <c r="K22" s="8" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="L22" s="12" t="inlineStr">
-        <is>
-          <t>높음</t>
-        </is>
-      </c>
-      <c r="M22" s="8" t="n">
-        <v>13</v>
-      </c>
-      <c r="N22" s="27" t="inlineStr">
-        <is>
-          <t>실제 사고 확인</t>
-        </is>
-      </c>
-      <c r="O22" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="P22" s="8" t="n">
-        <v>335</v>
-      </c>
-      <c r="Q22" s="8" t="inlineStr"/>
-      <c r="R22" s="9" t="inlineStr">
-        <is>
-          <t>■ 탐지
-- 로그 삭제·감사 정책 변경 이벤트와 원격 수집 로그의 공백을 모니터링(NIST AU-6·SI-4)
-■ 대응
-- 원격·불변 로그 전송과 로그 삭제 방지·보존 정책을 적용(NIST AU-9·AU-6)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>[DE] 방어 회피</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>ENT-DE-04</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>위장(정상 이름·서명)</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>위장(정상 이름·경로·서명 가장)</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>정상 이름·경로·서명 가장(위장)으로 눈·규칙 탐지 회피</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>- 공격자는 정상 프로세스·경로·서명으로 위장해 사람 눈과 규칙 기반 탐지를 피할 수 있음
-- 정상처럼 보여 레거시가 구분하기 어려우나 단독 피해는 제한적임</t>
-        </is>
-      </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>서명된 정상 도구 악용 · 시그니처 회피</t>
-        </is>
-      </c>
-      <c r="H23" s="8" t="inlineStr">
-        <is>
-          <t>EDR·XDR</t>
-        </is>
-      </c>
-      <c r="I23" s="9" t="inlineStr">
-        <is>
-          <t>Windows · Linux · macOS</t>
-        </is>
-      </c>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="K23" s="8" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="L23" s="13" t="inlineStr">
-        <is>
-          <t>보통</t>
-        </is>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>45</v>
-      </c>
-      <c r="N23" s="28" t="inlineStr">
-        <is>
-          <t>ATT&amp;CK 사례·KEV 다수</t>
-        </is>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="Q23" s="8" t="inlineStr"/>
-      <c r="R23" s="9" t="inlineStr">
-        <is>
-          <t>■ 탐지
-- 정상 이름과 다른 경로·서명·해시 불일치를 무결성·행위 기반으로 탐지(NIST SI-4·SI-7)
-■ 대응
-- 바이너리 무결성·서명 검증과 정상 경로 기준선 대조를 적용(NIST SI-7·SI-4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>[DE] 방어 회피</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>ENT-DE-05</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>파일·정보 난독화</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>파일·정보 난독화·암호화</t>
-        </is>
-      </c>
-      <c r="E24" s="9" t="inlineStr">
-        <is>
-          <t>패킹·인코딩·암호화 난독화로 시그니처·정적 분석 회피</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>- 공격자는 페이로드를 패킹·인코딩·암호화해 시그니처·정적 분석을 회피할 수 있음
-- 변종 양산으로 레거시 AV를 지속 우회하나 단독 피해는 제한적임</t>
-        </is>
-      </c>
-      <c r="G24" s="9" t="inlineStr">
-        <is>
-          <t>시그니처 회피 · 파일리스·인메모리</t>
-        </is>
-      </c>
-      <c r="H24" s="8" t="inlineStr">
-        <is>
-          <t>EDR·XDR</t>
-        </is>
-      </c>
-      <c r="I24" s="9" t="inlineStr">
-        <is>
-          <t>Windows · Linux · macOS</t>
-        </is>
-      </c>
-      <c r="J24" s="8" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="K24" s="8" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="L24" s="13" t="inlineStr">
-        <is>
-          <t>보통</t>
-        </is>
-      </c>
-      <c r="M24" s="8" t="n">
-        <v>40</v>
-      </c>
-      <c r="N24" s="28" t="inlineStr">
-        <is>
-          <t>ATT&amp;CK 사례·KEV 다수</t>
-        </is>
-      </c>
-      <c r="O24" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" s="8" t="n">
-        <v>160</v>
-      </c>
-      <c r="Q24" s="8" t="inlineStr"/>
-      <c r="R24" s="9" t="inlineStr">
-        <is>
-          <t>■ 탐지
-- 실행 시점 행위·언패킹과 비정상 인코딩·엔트로피를 행위 기반으로 탐지(NIST SI-3·SI-4)
-■ 대응
-- 시그니처 의존을 줄이고 행위 기반·샌드박스 분석을 병행(NIST SI-3·SI-4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>[DE] 방어 회피</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>ENT-DE-06</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>인메모리·반사 로딩</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>인메모리·반사 코드 로딩</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <t>인메모리·반사 코드 로딩으로 파일 기반 AV 원천 회피</t>
-        </is>
-      </c>
-      <c r="F25" s="9" t="inlineStr">
-        <is>
-          <t>- 공격자는 디스크를 거치지 않고 메모리에서 페이로드를 로드·실행할 수 있음
-- 파일 기반 AV·시그니처가 원천적으로 보지 못해 행위·메모리 기반 탐지가 필요함</t>
-        </is>
-      </c>
-      <c r="G25" s="9" t="inlineStr">
-        <is>
-          <t>파일리스·인메모리 · 시그니처 회피</t>
-        </is>
-      </c>
-      <c r="H25" s="8" t="inlineStr">
-        <is>
-          <t>행위·네트워크·아이덴티티</t>
-        </is>
-      </c>
-      <c r="I25" s="9" t="inlineStr">
-        <is>
-          <t>Windows</t>
-        </is>
-      </c>
-      <c r="J25" s="8" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="K25" s="8" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="L25" s="13" t="inlineStr">
-        <is>
-          <t>보통</t>
-        </is>
-      </c>
-      <c r="M25" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="N25" s="28" t="inlineStr">
-        <is>
-          <t>ATT&amp;CK 사례·KEV 다수</t>
-        </is>
-      </c>
-      <c r="O25" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" s="8" t="n">
-        <v>32</v>
-      </c>
-      <c r="Q25" s="8" t="inlineStr"/>
-      <c r="R25" s="9" t="inlineStr">
-        <is>
-          <t>■ 탐지
-- 메모리 영역 할당·실행과 비정상 로딩을 EDR 메모리 스캔으로 탐지(NIST SI-3·SI-4)
-■ 대응
-- 메모리 가시성(EDR)·공격 표면 축소와 스크립트 실행 통제를 적용(NIST SI-3·SI-4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>[DE] 방어 회피</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>ENT-DE-07</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>루트킷</t>
-        </is>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>루트킷(사용자·커널 은폐)</t>
-        </is>
-      </c>
-      <c r="E26" s="9" t="inlineStr">
-        <is>
-          <t>루트킷으로 프로세스·파일·연결을 하위 계층에서 은폐</t>
-        </is>
-      </c>
-      <c r="F26" s="9" t="inlineStr">
-        <is>
-          <t>- 공격자는 루트킷으로 프로세스·파일·연결을 하위 계층에서 숨겨 탐지·분석을 방해할 수 있음
-- 레거시로는 존재 자체를 알기 어려워 장기 잠복에 쓰임</t>
-        </is>
-      </c>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>커널·펌웨어 하위 계층 · 파일리스·인메모리</t>
-        </is>
-      </c>
-      <c r="H26" s="8" t="inlineStr">
-        <is>
-          <t>행위·네트워크·아이덴티티</t>
-        </is>
-      </c>
-      <c r="I26" s="9" t="inlineStr">
-        <is>
-          <t>Windows · Linux</t>
-        </is>
-      </c>
-      <c r="J26" s="8" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="K26" s="8" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="L26" s="13" t="inlineStr">
-        <is>
-          <t>보통</t>
-        </is>
-      </c>
-      <c r="M26" s="8" t="n">
-        <v>36</v>
-      </c>
-      <c r="N26" s="28" t="inlineStr">
-        <is>
-          <t>ATT&amp;CK 사례·KEV 다수</t>
-        </is>
-      </c>
-      <c r="O26" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" s="8" t="n">
-        <v>32</v>
-      </c>
-      <c r="Q26" s="8" t="inlineStr"/>
-      <c r="R26" s="9" t="inlineStr">
-        <is>
-          <t>■ 탐지
-- 커널 무결성·드라이버 서명과 메모리·부트 무결성 검증으로 은폐를 탐지(NIST SI-7·SI-4)
-■ 대응
-- 커널 무결성 보호(HVCI)·보안 부팅과 하위 계층 텔레메트리를 확보(NIST SI-7·SI-4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>[DE] 방어 회피</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>ENT-DE-08</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>펌웨어·부트 수준 은닉</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>펌웨어·부트킷(UEFI) 지속·은닉</t>
-        </is>
-      </c>
-      <c r="E27" s="9" t="inlineStr">
-        <is>
-          <t>펌웨어·부트킷(UEFI)으로 OS 아래 지속·은닉</t>
-        </is>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>- 공격자는 OS 아래 펌웨어·부트 단계에 임플란트를 심어 재설치·디스크 교체에도 지속할 수 있음
-- OS 보안 제품의 가시성 밖이라 레거시·EDR 모두 사실상 공백임</t>
-        </is>
-      </c>
-      <c r="G27" s="9" t="inlineStr">
-        <is>
-          <t>커널·펌웨어 하위 계층</t>
-        </is>
-      </c>
-      <c r="H27" s="8" t="inlineStr">
-        <is>
-          <t>행위·네트워크·아이덴티티</t>
-        </is>
-      </c>
-      <c r="I27" s="9" t="inlineStr">
-        <is>
-          <t>펌웨어 · Windows</t>
-        </is>
-      </c>
-      <c r="J27" s="8" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="K27" s="8" t="inlineStr">
-        <is>
-          <t>중</t>
-        </is>
-      </c>
-      <c r="L27" s="13" t="inlineStr">
-        <is>
-          <t>보통</t>
-        </is>
-      </c>
-      <c r="M27" s="8" t="n">
-        <v>26</v>
-      </c>
-      <c r="N27" s="27" t="inlineStr">
-        <is>
-          <t>실제 사고 확인</t>
-        </is>
-      </c>
-      <c r="O27" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="P27" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="8" t="inlineStr"/>
-      <c r="R27" s="9" t="inlineStr">
-        <is>
-          <t>■ 탐지
-- 펌웨어·부트 무결성 측정(보안 부팅·측정 부팅)과 펌웨어 버전·해시 변화를 점검(NIST SI-7)
-■ 대응
-- 보안 부팅·펌웨어 무결성 검증·업데이트와 펌웨어 공급 신뢰를 관리(NIST SI-7·CM-7)</t>
-        </is>
-      </c>
-    </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
@@ -20639,7 +20675,7 @@
       <c r="F34" s="9" t="inlineStr">
         <is>
           <t>- 공격자는 설치된 보안 제품을 확인해 회피·무력화를 준비할 수 있음
-- 사전 단계라 직접 피해는 없으나 이후 방어 회피로 이어짐</t>
+- 사전 단계라 직접 피해는 없으나 이후 은닉·방어 무력화로 이어짐</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
@@ -22350,7 +22386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -22678,30 +22714,30 @@
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>[DE] 방어 회피</t>
+          <t>[ST] 은닉</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>EDR 변조·BYOVD·지표 삭제·위장·난독화·인메모리·루트킷·펌웨어 — 레거시가 체계적으로 공백인 영역(ATT&amp;CK 미커버 148개 중 다수)</t>
+          <t>위장·난독화·암호화·인메모리·반사 로딩·루트킷·펌웨어·지표 삭제 — 정상 행위에 섞여 탐지를 피하는 영역(ATT&amp;CK v19 구 방어 회피 TA0005 유지)</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>클라우드 로그 무력화는 CL · AI 기반 적대적 회피는 AI(연계)</t>
+          <t>클라우드 로그 영역은 CL · AI 기반 적대적 회피는 AI(연계)</t>
         </is>
       </c>
       <c r="D6" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F6" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H6" s="9" t="n">
         <v>5</v>
@@ -22710,7 +22746,7 @@
         <v>0</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K6" s="9" t="n">
         <v>4</v>
@@ -22722,66 +22758,122 @@
         <v>0</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="O6" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-01.1 보안 도구 무력화(EDR 변조·BYOVD EDR 킬러)(높음)
-ENT-DE-01.2 취약·악성 드라이버 로드(커널)(높음)
-ENT-DE-03 지표 삭제(이벤트 로그·파일 삭제)(높음)</t>
+          <t>ENT-ST-01 지표 삭제(이벤트 로그·파일 삭제)(높음)
+ENT-ST-06 펌웨어·부트킷(UEFI) 지속·은닉(보통)
+ENT-ST-04 인메모리·반사 코드 로딩(보통)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>[CA] 자격증명 접근</t>
+          <t>[DM] 방어 무력화</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>LSASS 덤프·캐시 자격증명·Kerberoasting·입력 캡처로 호스트·도메인 자격증명을 탈취 — 이후 정상 인증으로 확산하는 발판</t>
+          <t>EDR 변조·BYOVD·취약 드라이버 로드 — 보안 통제를 직접 끄거나 떨어뜨리는 영역(ATT&amp;CK v19 신설 TA0112)</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>저장·노출된 비밀·토큰 재사용은 ID(연계)</t>
+          <t>클라우드 로그 무력화는 CL(연계) · AI 기반 적대적 회피는 AI(연계)</t>
         </is>
       </c>
       <c r="D7" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I7" s="9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7" s="9" t="n">
         <v>2</v>
       </c>
       <c r="K7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="O7" s="9" t="inlineStr">
+        <is>
+          <t>ENT-DM-01.1 보안 도구 무력화(EDR 변조·BYOVD EDR 킬러)(높음)
+ENT-DM-01.2 취약·악성 드라이버 로드(커널)(높음)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>[CA] 자격증명 접근</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>LSASS 덤프·캐시 자격증명·Kerberoasting·입력 캡처로 호스트·도메인 자격증명을 탈취 — 이후 정상 인증으로 확산하는 발판</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>저장·노출된 비밀·토큰 재사용은 ID(연계)</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="L7" s="9" t="n">
+      <c r="H8" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="M7" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="9" t="n">
+      <c r="J8" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="O7" s="9" t="inlineStr">
+      <c r="O8" s="9" t="inlineStr">
         <is>
           <t>ENT-CA-01.1 OS 자격증명 덤프(LSASS 메모리)(높음)
 ENT-CA-03 Kerberoasting·AS-REP 로스팅(보통)
@@ -22789,56 +22881,56 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>[DI] 탐색</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>호스트·네트워크·AD 열거로 표적·경로를 파악 — 정상 질의라 레거시가 공백(미커버 49개 중 38개)</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>클라우드 자원 탐색은 CL(연계)</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D9" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="E9" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="9" t="n">
+      <c r="F9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="9" t="n">
+      <c r="H9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="J8" s="9" t="n">
+      <c r="J9" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="K8" s="9" t="n">
+      <c r="K9" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="L8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="9" t="n">
+      <c r="L9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="O8" s="9" t="inlineStr">
+      <c r="O9" s="9" t="inlineStr">
         <is>
           <t>ENT-DI-02 도메인·AD 열거(계정·신뢰·공유)(높음)
 ENT-DI-01 호스트·시스템·네트워크 구성 탐색(높음)
@@ -22846,56 +22938,56 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>[LM] 측면 이동</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>원격 서비스·대체 인증 자료·도구 전송·원격 취약점으로 내부 확산 — 정상 프로토콜·인증을 써 레거시가 구분하기 어려움</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>토큰·티켓 위조 등 신원 전용은 ID(연계)</t>
         </is>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D10" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="E10" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="9" t="n">
+      <c r="F10" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="9" t="n">
+      <c r="G10" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H9" s="9" t="n">
+      <c r="H10" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="9" t="n">
+      <c r="I10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="K9" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="9" t="n">
+      <c r="K10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="O9" s="9" t="inlineStr">
+      <c r="O10" s="9" t="inlineStr">
         <is>
           <t>ENT-LM-04 원격 서비스 취약점 악용(웜 확산)(매우 높음)
 ENT-LM-01 원격 서비스 악용(RDP·SMB·WinRM)(높음)
@@ -22903,112 +22995,112 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>[CO] 수집</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>로컬·공유 데이터 수집과 스테이징 — 반출 전 단계</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>클라우드 스토리지·메일 수집은 CL(연계)</t>
         </is>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D11" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="9" t="n">
+      <c r="E11" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="9" t="n">
+      <c r="F11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="I10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="9" t="n">
+      <c r="I11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="L10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="9" t="inlineStr">
+      <c r="L11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="9" t="inlineStr">
         <is>
           <t>ENT-CO-01 로컬·네트워크 공유 데이터 수집(보통)
 ENT-CO-02 수집 데이터 압축·암호화 스테이징(보통)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>[C2] 명령·제어</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>암호화 채널·정상 포트·웹 서비스·도메인 프런팅·프록시·DNS로 통제 트래픽을 숨김 — 레거시가 거의 공백(미커버 45개 중 43개)</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>클라우드 서비스 경유 C2는 CL · AI 서비스 경유 C2는 AI(연계)</t>
         </is>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D12" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="E11" s="9" t="n">
+      <c r="E12" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="F11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="9" t="n">
+      <c r="F12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H11" s="9" t="n">
+      <c r="H12" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="I11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="9" t="n">
+      <c r="I12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="K11" s="9" t="n">
+      <c r="K12" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="L11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="9" t="n">
+      <c r="L12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="O11" s="9" t="inlineStr">
+      <c r="O12" s="9" t="inlineStr">
         <is>
           <t>ENT-C2-01.2 응용 계층 프로토콜(HTTPS) C2(높음)
 ENT-C2-05 인그레스 도구 전송(페이로드 반입)(높음)
@@ -23016,112 +23108,112 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>[EF] 반출</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>C2 채널·웹 서비스·대체 프로토콜로 데이터를 빼냄 — 정상 암호화 트래픽에 섞여 레거시 DLP·IDS가 놓침</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>클라우드 계정 간 전송·미러링 반출은 CL(연계)</t>
         </is>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D13" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="9" t="n">
+      <c r="E13" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F12" s="9" t="n">
+      <c r="F13" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="9" t="n">
+      <c r="G13" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="9" t="n">
+      <c r="H13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="K12" s="9" t="n">
+      <c r="K13" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="L12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="9" t="n">
+      <c r="L13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="O12" s="9" t="inlineStr">
+      <c r="O13" s="9" t="inlineStr">
         <is>
           <t>ENT-EF-02 정상 웹 서비스·대체 프로토콜 경유 반출(매우 높음)
 ENT-EF-01 C2 채널 경유 반출(높음)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>[IM] 영향</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>암호화(랜섬웨어)·복구 방해·파괴·서비스 중지·갈취 — 레거시가 막지 못한 침해의 최종 피해</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>클라우드·OT 영향은 CL·OT(연계)</t>
         </is>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D14" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="E13" s="9" t="n">
+      <c r="E14" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="F13" s="9" t="n">
+      <c r="F14" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="G13" s="9" t="n">
+      <c r="G14" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="9" t="n">
+      <c r="H14" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="I13" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="9" t="n">
+      <c r="I14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="K13" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="9" t="n">
+      <c r="K14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="O13" s="9" t="inlineStr">
+      <c r="O14" s="9" t="inlineStr">
         <is>
           <t>ENT-IM-01 데이터 암호화(사람 운영 랜섬웨어)(매우 높음)
 ENT-IM-05 금전 탈취·이중 협박 갈취(매우 높음)
@@ -23204,7 +23296,7 @@
       <c r="E4" s="9" t="inlineStr">
         <is>
           <t>ENT-LM-04 원격 서비스 취약점 악용(웜 확산)(매우 높음)
-ENT-DE-03 지표 삭제(이벤트 로그·파일 삭제)(높음)
+ENT-ST-01 지표 삭제(이벤트 로그·파일 삭제)(높음)
 ENT-EX-03 서명된 정상 바이너리 프록시 실행(LOLBin)(보통)</t>
         </is>
       </c>
@@ -23255,7 +23347,7 @@
         <is>
           <t>ENT-IM-01 데이터 암호화(사람 운영 랜섬웨어)(매우 높음)
 ENT-IM-02 복구 방해(섀도 카피·백업 삭제)(매우 높음)
-ENT-DE-01.1 보안 도구 무력화(EDR 변조·BYOVD EDR 킬러)(높음)</t>
+ENT-DM-01.1 보안 도구 무력화(EDR 변조·BYOVD EDR 킬러)(높음)</t>
         </is>
       </c>
     </row>
@@ -23353,8 +23445,8 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-01.1 보안 도구 무력화(EDR 변조·BYOVD EDR 킬러)(높음)
-ENT-DE-01.2 취약·악성 드라이버 로드(커널)(높음)
+          <t>ENT-DM-01.1 보안 도구 무력화(EDR 변조·BYOVD EDR 킬러)(높음)
+ENT-DM-01.2 취약·악성 드라이버 로드(커널)(높음)
 ENT-IM-03 데이터 파괴·와이퍼(높음)</t>
         </is>
       </c>
@@ -23705,12 +23797,12 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>방어 회피</t>
+          <t>방어 무력화</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-01.1, ENT-PV-04</t>
+          <t>ENT-DM-01.1, ENT-PV-04</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
@@ -24089,12 +24181,12 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>방어 회피</t>
+          <t>은닉</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-05, ENT-DE-04</t>
+          <t>ENT-ST-03, ENT-ST-02</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
@@ -24121,12 +24213,12 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>방어 회피</t>
+          <t>은닉</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-03</t>
+          <t>ENT-ST-01</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -24153,12 +24245,12 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>방어 회피</t>
+          <t>은닉</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-08</t>
+          <t>ENT-ST-06</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -24185,12 +24277,12 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>방어 회피</t>
+          <t>은닉</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-08</t>
+          <t>ENT-ST-06</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -24360,7 +24452,7 @@
       <c r="K2" s="9" t="inlineStr"/>
       <c r="L2" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-01.1, ENT-DE-01.2</t>
+          <t>ENT-DM-01.1, ENT-DM-01.2</t>
         </is>
       </c>
       <c r="M2" s="9" t="inlineStr"/>
@@ -24488,7 +24580,7 @@
       <c r="K4" s="9" t="inlineStr"/>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>ENT-IA-01, ENT-DE-03</t>
+          <t>ENT-IA-01, ENT-ST-01</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr"/>
@@ -24552,7 +24644,7 @@
       <c r="K5" s="9" t="inlineStr"/>
       <c r="L5" s="9" t="inlineStr">
         <is>
-          <t>ENT-IM-01, ENT-DE-01.1</t>
+          <t>ENT-IM-01, ENT-DM-01.1</t>
         </is>
       </c>
       <c r="M5" s="9" t="inlineStr"/>
@@ -24616,7 +24708,7 @@
       <c r="K6" s="9" t="inlineStr"/>
       <c r="L6" s="9" t="inlineStr">
         <is>
-          <t>ENT-IA-02, ENT-EX-03, ENT-CA-01.1, ENT-DI-02, ENT-DE-01.1, ENT-IM-02, ENT-IM-05</t>
+          <t>ENT-IA-02, ENT-EX-03, ENT-CA-01.1, ENT-DI-02, ENT-DM-01.1, ENT-IM-02, ENT-IM-05</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr"/>
@@ -24680,7 +24772,7 @@
       <c r="K7" s="9" t="inlineStr"/>
       <c r="L7" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-01.2, ENT-DE-01.1</t>
+          <t>ENT-DM-01.2, ENT-DM-01.1</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr"/>
@@ -24880,7 +24972,7 @@
       <c r="K10" s="9" t="inlineStr"/>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-01.1, ENT-DE-01.2, ENT-PV-04</t>
+          <t>ENT-DM-01.1, ENT-DM-01.2, ENT-PV-04</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
@@ -25016,7 +25108,7 @@
       <c r="K12" s="9" t="inlineStr"/>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>ENT-EX-01.1, ENT-CA-01.1, ENT-DI-02, ENT-LM-01, ENT-DE-01.1, ENT-IM-01, ENT-IM-02</t>
+          <t>ENT-EX-01.1, ENT-CA-01.1, ENT-DI-02, ENT-LM-01, ENT-DM-01.1, ENT-IM-01, ENT-IM-02</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
@@ -25356,7 +25448,7 @@
       <c r="K17" s="9" t="inlineStr"/>
       <c r="L17" s="9" t="inlineStr">
         <is>
-          <t>ENT-IA-01, ENT-EX-01.1, ENT-EX-03, ENT-DI-01, ENT-DI-02, ENT-CA-01.1, ENT-LM-01, ENT-DE-03</t>
+          <t>ENT-IA-01, ENT-EX-01.1, ENT-EX-03, ENT-DI-01, ENT-DI-02, ENT-CA-01.1, ENT-LM-01, ENT-ST-01</t>
         </is>
       </c>
       <c r="M17" s="9" t="inlineStr">
@@ -25492,7 +25584,7 @@
       <c r="K19" s="9" t="inlineStr"/>
       <c r="L19" s="9" t="inlineStr">
         <is>
-          <t>ENT-IA-02, ENT-DE-01.1, ENT-LM-01, ENT-LM-03, ENT-IM-01</t>
+          <t>ENT-IA-02, ENT-DM-01.1, ENT-LM-01, ENT-LM-03, ENT-IM-01</t>
         </is>
       </c>
       <c r="M19" s="9" t="inlineStr">
@@ -25760,7 +25852,7 @@
       <c r="K23" s="9" t="inlineStr"/>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>ENT-IM-01, ENT-IM-02, ENT-IM-04, ENT-DE-01.1</t>
+          <t>ENT-IM-01, ENT-IM-02, ENT-IM-04, ENT-DM-01.1</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr"/>
@@ -25893,7 +25985,7 @@
       <c r="K25" s="9" t="inlineStr"/>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-08</t>
+          <t>ENT-ST-06</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr"/>
@@ -25957,7 +26049,7 @@
       <c r="K26" s="9" t="inlineStr"/>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>ENT-DE-08</t>
+          <t>ENT-ST-06</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">

</xml_diff>